<commit_message>
Build ICPH form builder and FHIR workflow
</commit_message>
<xml_diff>
--- a/ODK/ODK XLSForm Template v2023.1.xlsx
+++ b/ODK/ODK XLSForm Template v2023.1.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="746" uniqueCount="449">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="733" uniqueCount="438">
   <si>
     <t>type</t>
   </si>
@@ -84,27 +84,6 @@
     <t>list_name</t>
   </si>
   <si>
-    <t>covered</t>
-  </si>
-  <si>
-    <t>yes</t>
-  </si>
-  <si>
-    <t>Yes (prescribed medications is covered in insurance)</t>
-  </si>
-  <si>
-    <t>no</t>
-  </si>
-  <si>
-    <t>No (prescribed medications are not covered in insurance)</t>
-  </si>
-  <si>
-    <t>unsure</t>
-  </si>
-  <si>
-    <t>Not sure (prescribed medications may / may not be covered in insurance)</t>
-  </si>
-  <si>
     <t>form_title</t>
   </si>
   <si>
@@ -121,18 +100,6 @@
   </si>
   <si>
     <t>style</t>
-  </si>
-  <si>
-    <t>Demo - Presciption claim and coverage info</t>
-  </si>
-  <si>
-    <t>demo_1</t>
-  </si>
-  <si>
-    <t>${patient_id}</t>
-  </si>
-  <si>
-    <t>english</t>
   </si>
   <si>
     <t xml:space="preserve"> Getting started with XLSForms</t>
@@ -16499,15 +16466,9 @@
       <c r="X498" s="6"/>
     </row>
   </sheetData>
-  <dataValidations count="4">
-    <dataValidation type="list" allowBlank="1" sqref="A10:A498">
-      <formula1>"'⚙️ Types'!$B$8:$B$46"</formula1>
-    </dataValidation>
+  <dataValidations count="2">
     <dataValidation type="list" allowBlank="1" sqref="A2:A498">
       <formula1>"'⚙️ Types'!$B$8:$B$46"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" sqref="G10:G498">
-      <formula1>"'👀 Appearances'!$B$7:$B$52"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" sqref="G2:G498">
       <formula1>"'👀 Appearances'!$B$7:$B$52"</formula1>
@@ -16537,7 +16498,7 @@
     <row r="1" ht="39" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1" s="103"/>
       <c r="B1" s="119" t="s">
-        <v>344</v>
+        <v>333</v>
       </c>
       <c r="C1" s="119"/>
       <c r="D1" s="119"/>
@@ -16561,7 +16522,7 @@
     <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" s="45"/>
       <c r="B3" s="45" t="s">
-        <v>345</v>
+        <v>334</v>
       </c>
       <c r="C3" s="45"/>
       <c r="D3" s="45"/>
@@ -16574,7 +16535,7 @@
     <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4" s="45"/>
       <c r="B4" s="45" t="s">
-        <v>346</v>
+        <v>335</v>
       </c>
       <c r="C4" s="45"/>
       <c r="D4" s="45"/>
@@ -16587,7 +16548,7 @@
     <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5" s="45"/>
       <c r="B5" s="45" t="s">
-        <v>347</v>
+        <v>336</v>
       </c>
       <c r="C5" s="45"/>
       <c r="D5" s="45"/>
@@ -16600,7 +16561,7 @@
     <row r="6" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A6" s="45"/>
       <c r="B6" s="45" t="s">
-        <v>348</v>
+        <v>337</v>
       </c>
       <c r="C6" s="45"/>
       <c r="D6" s="45"/>
@@ -16613,7 +16574,7 @@
     <row r="7" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A7" s="45"/>
       <c r="B7" s="45" t="s">
-        <v>349</v>
+        <v>338</v>
       </c>
       <c r="C7" s="45"/>
       <c r="D7" s="45"/>
@@ -16626,7 +16587,7 @@
     <row r="8" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A8" s="45"/>
       <c r="B8" s="45" t="s">
-        <v>350</v>
+        <v>339</v>
       </c>
       <c r="C8" s="45"/>
       <c r="D8" s="45"/>
@@ -16639,7 +16600,7 @@
     <row r="9" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A9" s="45"/>
       <c r="B9" s="45" t="s">
-        <v>351</v>
+        <v>340</v>
       </c>
       <c r="C9" s="45"/>
       <c r="D9" s="45"/>
@@ -16663,7 +16624,7 @@
     <row r="11" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A11" s="45"/>
       <c r="B11" s="37" t="s">
-        <v>352</v>
+        <v>341</v>
       </c>
       <c r="C11" s="45"/>
       <c r="D11" s="45"/>
@@ -16676,7 +16637,7 @@
     <row r="12" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A12" s="45"/>
       <c r="B12" s="13" t="s">
-        <v>353</v>
+        <v>342</v>
       </c>
       <c r="C12" s="13"/>
       <c r="D12" s="13"/>
@@ -16689,7 +16650,7 @@
     <row r="13" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A13" s="45"/>
       <c r="B13" s="121" t="s">
-        <v>354</v>
+        <v>343</v>
       </c>
       <c r="C13" s="45"/>
       <c r="D13" s="45"/>
@@ -16739,7 +16700,7 @@
     <row r="17" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A17" s="120"/>
       <c r="B17" s="124" t="s">
-        <v>355</v>
+        <v>344</v>
       </c>
       <c r="C17" s="54"/>
       <c r="D17" s="45"/>
@@ -16765,7 +16726,7 @@
     <row r="19" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A19" s="120"/>
       <c r="B19" s="124" t="s">
-        <v>356</v>
+        <v>345</v>
       </c>
       <c r="C19" s="54"/>
       <c r="D19" s="45"/>
@@ -16791,7 +16752,7 @@
     <row r="21" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A21" s="120"/>
       <c r="B21" s="124" t="s">
-        <v>135</v>
+        <v>124</v>
       </c>
       <c r="C21" s="54"/>
       <c r="D21" s="45"/>
@@ -16828,7 +16789,7 @@
     <row r="24" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A24" s="45"/>
       <c r="B24" s="37" t="s">
-        <v>357</v>
+        <v>346</v>
       </c>
       <c r="C24" s="45"/>
       <c r="D24" s="45"/>
@@ -16841,7 +16802,7 @@
     <row r="25" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A25" s="45"/>
       <c r="B25" s="45" t="s">
-        <v>358</v>
+        <v>347</v>
       </c>
       <c r="C25" s="45"/>
       <c r="D25" s="45"/>
@@ -16854,7 +16815,7 @@
     <row r="26" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A26" s="45"/>
       <c r="B26" s="47" t="s">
-        <v>359</v>
+        <v>348</v>
       </c>
       <c r="C26" s="45"/>
       <c r="D26" s="45"/>
@@ -16867,7 +16828,7 @@
     <row r="27" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A27" s="45"/>
       <c r="B27" s="48" t="s">
-        <v>360</v>
+        <v>349</v>
       </c>
       <c r="C27" s="45"/>
       <c r="D27" s="45"/>
@@ -16891,7 +16852,7 @@
     <row r="29" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A29" s="120"/>
       <c r="B29" s="127" t="s">
-        <v>361</v>
+        <v>350</v>
       </c>
       <c r="C29" s="54"/>
       <c r="D29" s="45"/>
@@ -16904,7 +16865,7 @@
     <row r="30" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A30" s="120"/>
       <c r="B30" s="125" t="s">
-        <v>362</v>
+        <v>351</v>
       </c>
       <c r="C30" s="54"/>
       <c r="D30" s="45"/>
@@ -16928,7 +16889,7 @@
     <row r="32" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A32" s="45"/>
       <c r="B32" s="37" t="s">
-        <v>363</v>
+        <v>352</v>
       </c>
       <c r="C32" s="45"/>
       <c r="D32" s="45"/>
@@ -16952,7 +16913,7 @@
     <row r="34" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A34" s="120"/>
       <c r="B34" s="128" t="s">
-        <v>364</v>
+        <v>353</v>
       </c>
       <c r="C34" s="129"/>
       <c r="D34" s="129"/>
@@ -16972,19 +16933,19 @@
         <v>1</v>
       </c>
       <c r="E35" s="9" t="s">
-        <v>365</v>
+        <v>354</v>
       </c>
       <c r="F35" s="10" t="s">
-        <v>361</v>
+        <v>350</v>
       </c>
       <c r="G35" s="9" t="s">
-        <v>366</v>
+        <v>355</v>
       </c>
       <c r="H35" s="10" t="s">
-        <v>362</v>
+        <v>351</v>
       </c>
       <c r="I35" s="9" t="s">
-        <v>367</v>
+        <v>356</v>
       </c>
     </row>
     <row r="36" spans="1:9" x14ac:dyDescent="0.25">
@@ -17001,7 +16962,7 @@
     <row r="37" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A37" s="120"/>
       <c r="B37" s="132" t="s">
-        <v>368</v>
+        <v>357</v>
       </c>
       <c r="C37" s="131"/>
       <c r="D37" s="131"/>
@@ -17021,16 +16982,16 @@
         <v>1</v>
       </c>
       <c r="E38" s="135" t="s">
-        <v>365</v>
+        <v>354</v>
       </c>
       <c r="F38" s="134" t="s">
-        <v>361</v>
+        <v>350</v>
       </c>
       <c r="G38" s="135" t="s">
-        <v>367</v>
+        <v>356</v>
       </c>
       <c r="H38" s="134" t="s">
-        <v>369</v>
+        <v>358</v>
       </c>
       <c r="I38" s="136"/>
     </row>
@@ -17086,7 +17047,7 @@
     <row r="1" ht="39" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="103"/>
       <c r="B1" s="119" t="s">
-        <v>370</v>
+        <v>359</v>
       </c>
       <c r="C1" s="119"/>
       <c r="D1" s="119"/>
@@ -17108,7 +17069,7 @@
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" s="45"/>
       <c r="B3" s="45" t="s">
-        <v>371</v>
+        <v>360</v>
       </c>
       <c r="C3" s="45"/>
       <c r="D3" s="45"/>
@@ -17120,7 +17081,7 @@
     <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" s="45"/>
       <c r="B4" s="138" t="s">
-        <v>372</v>
+        <v>361</v>
       </c>
       <c r="C4" s="45"/>
       <c r="D4" s="45"/>
@@ -17132,7 +17093,7 @@
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" s="45"/>
       <c r="B5" s="139" t="s">
-        <v>373</v>
+        <v>362</v>
       </c>
       <c r="C5" s="45"/>
       <c r="D5" s="45"/>
@@ -17154,7 +17115,7 @@
     <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" s="140"/>
       <c r="B7" s="141" t="s">
-        <v>374</v>
+        <v>363</v>
       </c>
       <c r="C7" s="142"/>
       <c r="D7" s="143"/>
@@ -17169,7 +17130,7 @@
         <v>19</v>
       </c>
       <c r="C8" s="145" t="s">
-        <v>375</v>
+        <v>364</v>
       </c>
       <c r="D8" s="146"/>
       <c r="E8" s="146"/>
@@ -17180,10 +17141,10 @@
     <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9" s="120"/>
       <c r="B9" s="147" t="s">
-        <v>376</v>
+        <v>365</v>
       </c>
       <c r="C9" s="148" t="s">
-        <v>377</v>
+        <v>366</v>
       </c>
       <c r="D9" s="149"/>
       <c r="E9" s="149"/>
@@ -17194,10 +17155,10 @@
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10" s="120"/>
       <c r="B10" s="150" t="s">
-        <v>378</v>
+        <v>367</v>
       </c>
       <c r="C10" s="148" t="s">
-        <v>379</v>
+        <v>368</v>
       </c>
       <c r="D10" s="149"/>
       <c r="E10" s="149"/>
@@ -17228,7 +17189,7 @@
     <row r="13" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A13" s="45"/>
       <c r="B13" s="37" t="s">
-        <v>380</v>
+        <v>369</v>
       </c>
       <c r="C13" s="45"/>
       <c r="D13" s="45"/>
@@ -17240,7 +17201,7 @@
     <row r="14" ht="24.75" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A14" s="48"/>
       <c r="B14" s="151" t="s">
-        <v>381</v>
+        <v>370</v>
       </c>
       <c r="C14" s="48"/>
       <c r="D14" s="48"/>
@@ -17252,7 +17213,7 @@
     <row r="15" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A15" s="152"/>
       <c r="B15" s="153" t="s">
-        <v>382</v>
+        <v>371</v>
       </c>
       <c r="C15" s="142"/>
       <c r="D15" s="143"/>
@@ -17267,7 +17228,7 @@
         <v>19</v>
       </c>
       <c r="C16" s="145" t="s">
-        <v>375</v>
+        <v>364</v>
       </c>
       <c r="D16" s="146"/>
       <c r="E16" s="146"/>
@@ -17278,10 +17239,10 @@
     <row r="17" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A17" s="154"/>
       <c r="B17" s="156" t="s">
-        <v>383</v>
+        <v>372</v>
       </c>
       <c r="C17" s="148" t="s">
-        <v>384</v>
+        <v>373</v>
       </c>
       <c r="D17" s="149"/>
       <c r="E17" s="149"/>
@@ -17292,10 +17253,10 @@
     <row r="18" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A18" s="154"/>
       <c r="B18" s="157" t="s">
-        <v>385</v>
+        <v>374</v>
       </c>
       <c r="C18" s="148" t="s">
-        <v>386</v>
+        <v>375</v>
       </c>
       <c r="D18" s="149"/>
       <c r="E18" s="149"/>
@@ -17306,10 +17267,10 @@
     <row r="19" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A19" s="158"/>
       <c r="B19" s="159" t="s">
-        <v>387</v>
+        <v>376</v>
       </c>
       <c r="C19" s="148" t="s">
-        <v>388</v>
+        <v>377</v>
       </c>
       <c r="D19" s="149"/>
       <c r="E19" s="149"/>
@@ -17330,112 +17291,112 @@
     <row r="21" ht="24.75" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A21" s="33"/>
       <c r="B21" s="162" t="s">
-        <v>389</v>
+        <v>378</v>
       </c>
       <c r="C21" s="163"/>
       <c r="D21" s="163"/>
       <c r="E21" s="163"/>
       <c r="F21" s="163"/>
       <c r="G21" s="164" t="s">
-        <v>86</v>
+        <v>75</v>
       </c>
       <c r="H21" s="36"/>
     </row>
     <row r="22" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A22" s="33"/>
       <c r="B22" s="165" t="s">
-        <v>390</v>
+        <v>379</v>
       </c>
       <c r="C22" s="165"/>
       <c r="D22" s="165"/>
       <c r="E22" s="165"/>
       <c r="F22" s="165"/>
       <c r="G22" s="166" t="s">
-        <v>391</v>
+        <v>380</v>
       </c>
       <c r="H22" s="36"/>
     </row>
     <row r="23" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A23" s="33"/>
       <c r="B23" s="167" t="s">
-        <v>392</v>
+        <v>381</v>
       </c>
       <c r="C23" s="167"/>
       <c r="D23" s="167"/>
       <c r="E23" s="167"/>
       <c r="F23" s="167"/>
       <c r="G23" s="168" t="s">
-        <v>393</v>
+        <v>382</v>
       </c>
       <c r="H23" s="36"/>
     </row>
     <row r="24" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A24" s="33"/>
       <c r="B24" s="165" t="s">
-        <v>394</v>
+        <v>383</v>
       </c>
       <c r="C24" s="165"/>
       <c r="D24" s="165"/>
       <c r="E24" s="165"/>
       <c r="F24" s="165"/>
       <c r="G24" s="166" t="s">
-        <v>395</v>
+        <v>384</v>
       </c>
       <c r="H24" s="36"/>
     </row>
     <row r="25" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A25" s="169"/>
       <c r="B25" s="167" t="s">
-        <v>396</v>
+        <v>385</v>
       </c>
       <c r="C25" s="167"/>
       <c r="D25" s="167"/>
       <c r="E25" s="167"/>
       <c r="F25" s="167"/>
       <c r="G25" s="168" t="s">
-        <v>397</v>
+        <v>386</v>
       </c>
       <c r="H25" s="36"/>
     </row>
     <row r="26" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A26" s="33"/>
       <c r="B26" s="165" t="s">
-        <v>398</v>
+        <v>387</v>
       </c>
       <c r="C26" s="165"/>
       <c r="D26" s="165"/>
       <c r="E26" s="165"/>
       <c r="F26" s="165"/>
       <c r="G26" s="166" t="s">
-        <v>399</v>
+        <v>388</v>
       </c>
       <c r="H26" s="36"/>
     </row>
     <row r="27" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A27" s="33"/>
       <c r="B27" s="167" t="s">
-        <v>400</v>
+        <v>389</v>
       </c>
       <c r="C27" s="167"/>
       <c r="D27" s="167"/>
       <c r="E27" s="167"/>
       <c r="F27" s="167"/>
       <c r="G27" s="168" t="s">
-        <v>401</v>
+        <v>390</v>
       </c>
       <c r="H27" s="36"/>
     </row>
     <row r="28" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A28" s="33"/>
       <c r="B28" s="170" t="s">
-        <v>402</v>
+        <v>391</v>
       </c>
       <c r="C28" s="171"/>
       <c r="D28" s="171"/>
       <c r="E28" s="171"/>
       <c r="F28" s="171"/>
       <c r="G28" s="172" t="s">
-        <v>403</v>
+        <v>392</v>
       </c>
       <c r="H28" s="36"/>
     </row>
@@ -17452,7 +17413,7 @@
     <row r="30" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A30" s="33"/>
       <c r="B30" s="149" t="s">
-        <v>404</v>
+        <v>393</v>
       </c>
       <c r="C30" s="149"/>
       <c r="D30" s="149"/>
@@ -17464,7 +17425,7 @@
     <row r="31" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A31" s="33"/>
       <c r="B31" s="149" t="s">
-        <v>405</v>
+        <v>394</v>
       </c>
       <c r="C31" s="149"/>
       <c r="D31" s="149"/>
@@ -17486,7 +17447,7 @@
     <row r="33" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A33" s="16"/>
       <c r="B33" s="173" t="s">
-        <v>406</v>
+        <v>395</v>
       </c>
       <c r="C33" s="173"/>
       <c r="D33" s="173"/>
@@ -17498,7 +17459,7 @@
     <row r="34" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A34" s="174"/>
       <c r="B34" s="149" t="s">
-        <v>407</v>
+        <v>396</v>
       </c>
       <c r="C34" s="149"/>
       <c r="D34" s="149"/>
@@ -17520,7 +17481,7 @@
     <row r="36" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A36" s="16"/>
       <c r="B36" s="149" t="s">
-        <v>408</v>
+        <v>397</v>
       </c>
       <c r="C36" s="149"/>
       <c r="D36" s="149"/>
@@ -17532,7 +17493,7 @@
     <row r="37" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A37" s="174"/>
       <c r="B37" s="149" t="s">
-        <v>409</v>
+        <v>398</v>
       </c>
       <c r="C37" s="149"/>
       <c r="D37" s="149"/>
@@ -17584,7 +17545,7 @@
     <row r="1" ht="33" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="176"/>
       <c r="B1" s="119" t="s">
-        <v>410</v>
+        <v>399</v>
       </c>
       <c r="C1" s="119"/>
       <c r="D1" s="119"/>
@@ -17606,7 +17567,7 @@
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" s="35"/>
       <c r="B3" s="35" t="s">
-        <v>411</v>
+        <v>400</v>
       </c>
       <c r="C3" s="35"/>
       <c r="D3" s="35"/>
@@ -17628,18 +17589,18 @@
     <row r="5" ht="21.75" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" s="178"/>
       <c r="B5" s="179" t="s">
-        <v>412</v>
+        <v>401</v>
       </c>
       <c r="C5" s="180"/>
       <c r="D5" s="181"/>
       <c r="E5" s="85" t="s">
-        <v>87</v>
+        <v>76</v>
       </c>
       <c r="F5" s="85" t="s">
-        <v>88</v>
+        <v>77</v>
       </c>
       <c r="G5" s="182" t="s">
-        <v>413</v>
+        <v>402</v>
       </c>
       <c r="H5" s="183"/>
     </row>
@@ -17647,19 +17608,19 @@
       <c r="A6" s="178"/>
       <c r="B6" s="184"/>
       <c r="C6" s="185" t="s">
-        <v>414</v>
+        <v>403</v>
       </c>
       <c r="D6" s="186" t="s">
-        <v>415</v>
+        <v>404</v>
       </c>
       <c r="E6" s="187" t="s">
-        <v>92</v>
+        <v>81</v>
       </c>
       <c r="F6" s="187" t="s">
-        <v>92</v>
+        <v>81</v>
       </c>
       <c r="G6" s="188" t="s">
-        <v>242</v>
+        <v>231</v>
       </c>
       <c r="H6" s="183"/>
     </row>
@@ -17667,19 +17628,19 @@
       <c r="A7" s="178"/>
       <c r="B7" s="189"/>
       <c r="C7" s="190" t="s">
-        <v>355</v>
+        <v>344</v>
       </c>
       <c r="D7" s="191" t="s">
-        <v>416</v>
+        <v>405</v>
       </c>
       <c r="E7" s="192" t="s">
-        <v>92</v>
+        <v>81</v>
       </c>
       <c r="F7" s="193" t="s">
-        <v>92</v>
+        <v>81</v>
       </c>
       <c r="G7" s="194" t="s">
-        <v>92</v>
+        <v>81</v>
       </c>
       <c r="H7" s="183"/>
     </row>
@@ -17687,19 +17648,19 @@
       <c r="A8" s="178"/>
       <c r="B8" s="184"/>
       <c r="C8" s="185" t="s">
-        <v>356</v>
+        <v>345</v>
       </c>
       <c r="D8" s="185" t="s">
-        <v>417</v>
+        <v>406</v>
       </c>
       <c r="E8" s="187" t="s">
-        <v>92</v>
+        <v>81</v>
       </c>
       <c r="F8" s="187" t="s">
-        <v>92</v>
+        <v>81</v>
       </c>
       <c r="G8" s="195" t="s">
-        <v>92</v>
+        <v>81</v>
       </c>
       <c r="H8" s="183"/>
     </row>
@@ -17707,19 +17668,19 @@
       <c r="A9" s="178"/>
       <c r="B9" s="189"/>
       <c r="C9" s="190" t="s">
-        <v>418</v>
+        <v>407</v>
       </c>
       <c r="D9" s="190" t="s">
-        <v>419</v>
+        <v>408</v>
       </c>
       <c r="E9" s="193" t="s">
-        <v>92</v>
+        <v>81</v>
       </c>
       <c r="F9" s="196" t="s">
-        <v>420</v>
+        <v>409</v>
       </c>
       <c r="G9" s="188" t="s">
-        <v>242</v>
+        <v>231</v>
       </c>
       <c r="H9" s="183"/>
     </row>
@@ -17727,19 +17688,19 @@
       <c r="A10" s="178"/>
       <c r="B10" s="184"/>
       <c r="C10" s="185" t="s">
-        <v>421</v>
+        <v>410</v>
       </c>
       <c r="D10" s="185" t="s">
-        <v>422</v>
+        <v>411</v>
       </c>
       <c r="E10" s="187" t="s">
-        <v>92</v>
+        <v>81</v>
       </c>
       <c r="F10" s="187" t="s">
-        <v>92</v>
+        <v>81</v>
       </c>
       <c r="G10" s="188" t="s">
-        <v>92</v>
+        <v>81</v>
       </c>
       <c r="H10" s="183"/>
     </row>
@@ -17747,19 +17708,19 @@
       <c r="A11" s="197"/>
       <c r="B11" s="189"/>
       <c r="C11" s="190" t="s">
-        <v>423</v>
+        <v>412</v>
       </c>
       <c r="D11" s="190" t="s">
-        <v>424</v>
+        <v>413</v>
       </c>
       <c r="E11" s="193" t="s">
-        <v>92</v>
+        <v>81</v>
       </c>
       <c r="F11" s="193" t="s">
-        <v>92</v>
+        <v>81</v>
       </c>
       <c r="G11" s="188" t="s">
-        <v>242</v>
+        <v>231</v>
       </c>
       <c r="H11" s="183"/>
     </row>
@@ -17767,19 +17728,19 @@
       <c r="A12" s="178"/>
       <c r="B12" s="184"/>
       <c r="C12" s="185" t="s">
-        <v>425</v>
+        <v>414</v>
       </c>
       <c r="D12" s="185" t="s">
-        <v>426</v>
+        <v>415</v>
       </c>
       <c r="E12" s="187" t="s">
-        <v>92</v>
+        <v>81</v>
       </c>
       <c r="F12" s="187" t="s">
-        <v>92</v>
+        <v>81</v>
       </c>
       <c r="G12" s="188" t="s">
-        <v>242</v>
+        <v>231</v>
       </c>
       <c r="H12" s="183"/>
     </row>
@@ -17787,19 +17748,19 @@
       <c r="A13" s="197"/>
       <c r="B13" s="198"/>
       <c r="C13" s="199" t="s">
-        <v>427</v>
+        <v>416</v>
       </c>
       <c r="D13" s="199" t="s">
-        <v>428</v>
+        <v>417</v>
       </c>
       <c r="E13" s="200" t="s">
-        <v>92</v>
+        <v>81</v>
       </c>
       <c r="F13" s="200" t="s">
-        <v>92</v>
+        <v>81</v>
       </c>
       <c r="G13" s="201" t="s">
-        <v>242</v>
+        <v>231</v>
       </c>
       <c r="H13" s="183"/>
     </row>
@@ -17816,7 +17777,7 @@
     <row r="15" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A15" s="178"/>
       <c r="B15" s="179" t="s">
-        <v>429</v>
+        <v>418</v>
       </c>
       <c r="C15" s="204"/>
       <c r="D15" s="204"/>
@@ -17832,16 +17793,16 @@
         <v>16</v>
       </c>
       <c r="D16" s="185" t="s">
-        <v>430</v>
+        <v>419</v>
       </c>
       <c r="E16" s="187" t="s">
-        <v>92</v>
+        <v>81</v>
       </c>
       <c r="F16" s="187" t="s">
-        <v>92</v>
+        <v>81</v>
       </c>
       <c r="G16" s="195" t="s">
-        <v>92</v>
+        <v>81</v>
       </c>
       <c r="H16" s="183"/>
     </row>
@@ -17849,19 +17810,19 @@
       <c r="A17" s="178"/>
       <c r="B17" s="184"/>
       <c r="C17" s="185" t="s">
-        <v>135</v>
+        <v>124</v>
       </c>
       <c r="D17" s="185" t="s">
-        <v>431</v>
+        <v>420</v>
       </c>
       <c r="E17" s="187" t="s">
-        <v>92</v>
+        <v>81</v>
       </c>
       <c r="F17" s="187" t="s">
-        <v>92</v>
+        <v>81</v>
       </c>
       <c r="G17" s="195" t="s">
-        <v>92</v>
+        <v>81</v>
       </c>
       <c r="H17" s="183"/>
     </row>
@@ -17872,16 +17833,16 @@
         <v>18</v>
       </c>
       <c r="D18" s="185" t="s">
-        <v>432</v>
+        <v>421</v>
       </c>
       <c r="E18" s="187" t="s">
-        <v>92</v>
+        <v>81</v>
       </c>
       <c r="F18" s="187" t="s">
-        <v>92</v>
+        <v>81</v>
       </c>
       <c r="G18" s="195" t="s">
-        <v>92</v>
+        <v>81</v>
       </c>
       <c r="H18" s="183"/>
     </row>
@@ -17889,19 +17850,19 @@
       <c r="A19" s="178"/>
       <c r="B19" s="206"/>
       <c r="C19" s="207" t="s">
-        <v>433</v>
+        <v>422</v>
       </c>
       <c r="D19" s="208" t="s">
-        <v>434</v>
+        <v>423</v>
       </c>
       <c r="E19" s="209" t="s">
-        <v>92</v>
+        <v>81</v>
       </c>
       <c r="F19" s="209" t="s">
-        <v>134</v>
+        <v>123</v>
       </c>
       <c r="G19" s="201" t="s">
-        <v>242</v>
+        <v>231</v>
       </c>
       <c r="H19" s="183"/>
     </row>
@@ -17917,7 +17878,7 @@
     <row r="21" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A21" s="178"/>
       <c r="B21" s="210" t="s">
-        <v>435</v>
+        <v>424</v>
       </c>
       <c r="C21" s="211"/>
       <c r="D21" s="211"/>
@@ -17930,19 +17891,19 @@
       <c r="A22" s="178"/>
       <c r="B22" s="213"/>
       <c r="C22" s="214" t="s">
-        <v>436</v>
+        <v>425</v>
       </c>
       <c r="D22" s="214" t="s">
-        <v>437</v>
+        <v>426</v>
       </c>
       <c r="E22" s="215" t="s">
-        <v>92</v>
+        <v>81</v>
       </c>
       <c r="F22" s="215" t="s">
-        <v>92</v>
+        <v>81</v>
       </c>
       <c r="G22" s="216" t="s">
-        <v>242</v>
+        <v>231</v>
       </c>
       <c r="H22" s="183"/>
     </row>
@@ -17950,19 +17911,19 @@
       <c r="A23" s="178"/>
       <c r="B23" s="184"/>
       <c r="C23" s="185" t="s">
-        <v>438</v>
+        <v>427</v>
       </c>
       <c r="D23" s="185" t="s">
-        <v>439</v>
+        <v>428</v>
       </c>
       <c r="E23" s="187" t="s">
-        <v>92</v>
+        <v>81</v>
       </c>
       <c r="F23" s="187" t="s">
-        <v>134</v>
+        <v>123</v>
       </c>
       <c r="G23" s="216" t="s">
-        <v>242</v>
+        <v>231</v>
       </c>
       <c r="H23" s="183"/>
     </row>
@@ -17970,19 +17931,19 @@
       <c r="A24" s="178"/>
       <c r="B24" s="206"/>
       <c r="C24" s="207" t="s">
-        <v>440</v>
+        <v>429</v>
       </c>
       <c r="D24" s="208" t="s">
-        <v>441</v>
+        <v>430</v>
       </c>
       <c r="E24" s="209" t="s">
-        <v>92</v>
+        <v>81</v>
       </c>
       <c r="F24" s="209" t="s">
-        <v>92</v>
+        <v>81</v>
       </c>
       <c r="G24" s="217" t="s">
-        <v>242</v>
+        <v>231</v>
       </c>
       <c r="H24" s="218"/>
     </row>
@@ -17999,7 +17960,7 @@
     <row r="26" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A26" s="178"/>
       <c r="B26" s="210" t="s">
-        <v>442</v>
+        <v>431</v>
       </c>
       <c r="C26" s="211"/>
       <c r="D26" s="211"/>
@@ -18012,19 +17973,19 @@
       <c r="A27" s="178"/>
       <c r="B27" s="221"/>
       <c r="C27" s="185" t="s">
-        <v>443</v>
+        <v>432</v>
       </c>
       <c r="D27" s="185" t="s">
-        <v>444</v>
+        <v>433</v>
       </c>
       <c r="E27" s="187" t="s">
-        <v>92</v>
+        <v>81</v>
       </c>
       <c r="F27" s="187" t="s">
-        <v>92</v>
+        <v>81</v>
       </c>
       <c r="G27" s="216" t="s">
-        <v>242</v>
+        <v>231</v>
       </c>
       <c r="H27" s="183"/>
     </row>
@@ -18032,19 +17993,19 @@
       <c r="A28" s="178"/>
       <c r="B28" s="221"/>
       <c r="C28" s="185" t="s">
-        <v>445</v>
+        <v>434</v>
       </c>
       <c r="D28" s="185" t="s">
-        <v>446</v>
+        <v>435</v>
       </c>
       <c r="E28" s="187" t="s">
-        <v>92</v>
+        <v>81</v>
       </c>
       <c r="F28" s="187" t="s">
-        <v>92</v>
+        <v>81</v>
       </c>
       <c r="G28" s="216" t="s">
-        <v>242</v>
+        <v>231</v>
       </c>
       <c r="H28" s="183"/>
     </row>
@@ -18052,19 +18013,19 @@
       <c r="A29" s="178"/>
       <c r="B29" s="222"/>
       <c r="C29" s="223" t="s">
-        <v>447</v>
+        <v>436</v>
       </c>
       <c r="D29" s="223" t="s">
-        <v>448</v>
+        <v>437</v>
       </c>
       <c r="E29" s="224" t="s">
-        <v>92</v>
+        <v>81</v>
       </c>
       <c r="F29" s="224" t="s">
-        <v>92</v>
+        <v>81</v>
       </c>
       <c r="G29" s="201" t="s">
-        <v>242</v>
+        <v>231</v>
       </c>
       <c r="H29" s="183"/>
     </row>
@@ -18116,15 +18077,9 @@
       <c r="H1" s="10"/>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A2" s="11" t="s">
-        <v>20</v>
-      </c>
-      <c r="B2" s="12" t="s">
-        <v>21</v>
-      </c>
-      <c r="C2" s="11" t="s">
-        <v>22</v>
-      </c>
+      <c r="A2" s="11"/>
+      <c r="B2" s="12"/>
+      <c r="C2" s="11"/>
       <c r="D2" s="13"/>
       <c r="E2" s="13"/>
       <c r="F2" s="13"/>
@@ -18132,15 +18087,9 @@
       <c r="H2" s="13"/>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A3" s="11" t="s">
-        <v>20</v>
-      </c>
-      <c r="B3" s="12" t="s">
-        <v>23</v>
-      </c>
-      <c r="C3" s="11" t="s">
-        <v>24</v>
-      </c>
+      <c r="A3" s="11"/>
+      <c r="B3" s="12"/>
+      <c r="C3" s="11"/>
       <c r="D3" s="13"/>
       <c r="E3" s="13"/>
       <c r="F3" s="13"/>
@@ -18148,15 +18097,9 @@
       <c r="H3" s="13"/>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A4" s="11" t="s">
-        <v>20</v>
-      </c>
-      <c r="B4" s="12" t="s">
-        <v>25</v>
-      </c>
-      <c r="C4" s="11" t="s">
-        <v>26</v>
-      </c>
+      <c r="A4" s="11"/>
+      <c r="B4" s="12"/>
+      <c r="C4" s="11"/>
       <c r="D4" s="13"/>
       <c r="E4" s="13"/>
       <c r="F4" s="13"/>
@@ -23121,7 +23064,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:M499"/>
+  <dimension ref="A1:M498"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="25.571428571428573" customWidth="1"/>
@@ -23134,22 +23077,22 @@
   <sheetData>
     <row r="1" ht="25.5" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A1" s="14" t="s">
-        <v>27</v>
+        <v>20</v>
       </c>
       <c r="B1" s="14" t="s">
-        <v>28</v>
+        <v>21</v>
       </c>
       <c r="C1" s="14" t="s">
-        <v>29</v>
+        <v>22</v>
       </c>
       <c r="D1" s="14" t="s">
-        <v>30</v>
+        <v>23</v>
       </c>
       <c r="E1" s="14" t="s">
-        <v>31</v>
+        <v>24</v>
       </c>
       <c r="F1" s="14" t="s">
-        <v>32</v>
+        <v>25</v>
       </c>
       <c r="G1" s="15"/>
       <c r="H1" s="15"/>
@@ -23160,21 +23103,11 @@
       <c r="M1" s="15"/>
     </row>
     <row r="2" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A2" s="13" t="s">
-        <v>33</v>
-      </c>
-      <c r="B2" s="13" t="s">
-        <v>34</v>
-      </c>
-      <c r="C2" s="13">
-        <f>TEXT(NOW(), "yyyymmddhhmmss")</f>
-      </c>
-      <c r="D2" s="13" t="s">
-        <v>35</v>
-      </c>
-      <c r="E2" s="13" t="s">
-        <v>36</v>
-      </c>
+      <c r="A2" s="13"/>
+      <c r="B2" s="13"/>
+      <c r="C2" s="13"/>
+      <c r="D2" s="13"/>
+      <c r="E2" s="13"/>
       <c r="F2" s="13"/>
       <c r="G2" s="13"/>
       <c r="H2" s="13"/>
@@ -30623,21 +30556,6 @@
       <c r="K498" s="13"/>
       <c r="L498" s="13"/>
       <c r="M498" s="13"/>
-    </row>
-    <row r="499" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A499" s="13"/>
-      <c r="B499" s="13"/>
-      <c r="C499" s="13"/>
-      <c r="D499" s="13"/>
-      <c r="E499" s="13"/>
-      <c r="F499" s="13"/>
-      <c r="G499" s="13"/>
-      <c r="H499" s="13"/>
-      <c r="I499" s="13"/>
-      <c r="J499" s="13"/>
-      <c r="K499" s="13"/>
-      <c r="L499" s="13"/>
-      <c r="M499" s="13"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -35174,17 +35092,17 @@
       <c r="A1" s="16"/>
       <c r="B1" s="17"/>
       <c r="C1" s="18" t="s">
-        <v>37</v>
+        <v>26</v>
       </c>
       <c r="D1" s="18"/>
       <c r="E1" s="16"/>
       <c r="F1" s="16"/>
       <c r="G1" s="19"/>
       <c r="H1" s="20" t="s">
-        <v>38</v>
+        <v>27</v>
       </c>
       <c r="I1" s="19" t="s">
-        <v>39</v>
+        <v>28</v>
       </c>
       <c r="J1" s="16"/>
     </row>
@@ -35197,10 +35115,10 @@
       <c r="F2" s="21"/>
       <c r="G2" s="22"/>
       <c r="H2" s="23" t="s">
-        <v>40</v>
+        <v>29</v>
       </c>
       <c r="I2" s="22" t="s">
-        <v>41</v>
+        <v>30</v>
       </c>
       <c r="J2" s="16"/>
     </row>
@@ -35219,7 +35137,7 @@
     <row r="4" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A4" s="16"/>
       <c r="B4" s="29" t="s">
-        <v>42</v>
+        <v>31</v>
       </c>
       <c r="C4" s="30"/>
       <c r="D4" s="30"/>
@@ -35233,7 +35151,7 @@
     <row r="5" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A5" s="16"/>
       <c r="B5" s="32" t="s">
-        <v>43</v>
+        <v>32</v>
       </c>
       <c r="C5" s="32"/>
       <c r="D5" s="32"/>
@@ -35247,7 +35165,7 @@
     <row r="6" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A6" s="33"/>
       <c r="B6" s="34" t="s">
-        <v>44</v>
+        <v>33</v>
       </c>
       <c r="C6" s="35"/>
       <c r="D6" s="16"/>
@@ -35261,7 +35179,7 @@
     <row r="7" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A7" s="33"/>
       <c r="B7" s="16" t="s">
-        <v>45</v>
+        <v>34</v>
       </c>
       <c r="C7" s="35"/>
       <c r="D7" s="16"/>
@@ -35275,7 +35193,7 @@
     <row r="8" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A8" s="33"/>
       <c r="B8" s="16" t="s">
-        <v>46</v>
+        <v>35</v>
       </c>
       <c r="C8" s="35"/>
       <c r="D8" s="16"/>
@@ -35289,7 +35207,7 @@
     <row r="9" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A9" s="33"/>
       <c r="B9" s="16" t="s">
-        <v>47</v>
+        <v>36</v>
       </c>
       <c r="C9" s="35"/>
       <c r="D9" s="16"/>
@@ -35315,7 +35233,7 @@
     <row r="11" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A11" s="16"/>
       <c r="B11" s="25" t="s">
-        <v>48</v>
+        <v>37</v>
       </c>
       <c r="C11" s="25"/>
       <c r="D11" s="25"/>
@@ -35329,7 +35247,7 @@
     <row r="12" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A12" s="16"/>
       <c r="B12" s="16" t="s">
-        <v>49</v>
+        <v>38</v>
       </c>
       <c r="C12" s="16"/>
       <c r="D12" s="16"/>
@@ -35343,7 +35261,7 @@
     <row r="13" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A13" s="16"/>
       <c r="B13" s="16" t="s">
-        <v>50</v>
+        <v>39</v>
       </c>
       <c r="C13" s="16"/>
       <c r="D13" s="16"/>
@@ -35369,7 +35287,7 @@
     <row r="15" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A15" s="16"/>
       <c r="B15" s="16" t="s">
-        <v>51</v>
+        <v>40</v>
       </c>
       <c r="C15" s="16"/>
       <c r="D15" s="16"/>
@@ -35383,7 +35301,7 @@
     <row r="16" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A16" s="16"/>
       <c r="B16" s="16" t="s">
-        <v>52</v>
+        <v>41</v>
       </c>
       <c r="C16" s="16"/>
       <c r="D16" s="16"/>
@@ -35397,7 +35315,7 @@
     <row r="17" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A17" s="16"/>
       <c r="B17" s="16" t="s">
-        <v>53</v>
+        <v>42</v>
       </c>
       <c r="C17" s="16"/>
       <c r="D17" s="16"/>
@@ -35423,7 +35341,7 @@
     <row r="19" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A19" s="16"/>
       <c r="B19" s="37" t="s">
-        <v>54</v>
+        <v>43</v>
       </c>
       <c r="C19" s="37"/>
       <c r="D19" s="16"/>
@@ -35437,7 +35355,7 @@
     <row r="20" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A20" s="16"/>
       <c r="B20" s="38" t="s">
-        <v>55</v>
+        <v>44</v>
       </c>
       <c r="C20" s="16"/>
       <c r="D20" s="16"/>
@@ -35451,7 +35369,7 @@
     <row r="21" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A21" s="16"/>
       <c r="B21" s="38" t="s">
-        <v>56</v>
+        <v>45</v>
       </c>
       <c r="C21" s="16"/>
       <c r="D21" s="16"/>
@@ -35465,7 +35383,7 @@
     <row r="22" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A22" s="16"/>
       <c r="B22" s="39" t="s">
-        <v>57</v>
+        <v>46</v>
       </c>
       <c r="C22" s="16"/>
       <c r="D22" s="16"/>
@@ -35479,7 +35397,7 @@
     <row r="23" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A23" s="16"/>
       <c r="B23" s="38" t="s">
-        <v>58</v>
+        <v>47</v>
       </c>
       <c r="C23" s="16"/>
       <c r="D23" s="16"/>
@@ -35505,7 +35423,7 @@
     <row r="25" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A25" s="16"/>
       <c r="B25" s="40" t="s">
-        <v>59</v>
+        <v>48</v>
       </c>
       <c r="C25" s="16"/>
       <c r="D25" s="16"/>
@@ -35519,7 +35437,7 @@
     <row r="26" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A26" s="16"/>
       <c r="B26" s="39" t="s">
-        <v>60</v>
+        <v>49</v>
       </c>
       <c r="C26" s="16"/>
       <c r="D26" s="16"/>
@@ -35533,7 +35451,7 @@
     <row r="27" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A27" s="16"/>
       <c r="B27" s="39" t="s">
-        <v>61</v>
+        <v>50</v>
       </c>
       <c r="C27" s="16"/>
       <c r="D27" s="16"/>
@@ -35559,7 +35477,7 @@
     <row r="29" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A29" s="16"/>
       <c r="B29" s="40" t="s">
-        <v>62</v>
+        <v>51</v>
       </c>
       <c r="C29" s="16"/>
       <c r="D29" s="16"/>
@@ -35573,10 +35491,10 @@
     <row r="30" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A30" s="16"/>
       <c r="B30" s="42" t="s">
-        <v>40</v>
+        <v>29</v>
       </c>
       <c r="C30" s="16" t="s">
-        <v>63</v>
+        <v>52</v>
       </c>
       <c r="D30" s="16"/>
       <c r="E30" s="16"/>
@@ -35589,10 +35507,10 @@
     <row r="31" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A31" s="16"/>
       <c r="B31" s="42" t="s">
-        <v>64</v>
+        <v>53</v>
       </c>
       <c r="C31" s="16" t="s">
-        <v>65</v>
+        <v>54</v>
       </c>
       <c r="D31" s="16"/>
       <c r="E31" s="16"/>
@@ -35605,10 +35523,10 @@
     <row r="32" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A32" s="16"/>
       <c r="B32" s="42" t="s">
-        <v>66</v>
+        <v>55</v>
       </c>
       <c r="C32" s="16" t="s">
-        <v>67</v>
+        <v>56</v>
       </c>
       <c r="D32" s="16"/>
       <c r="E32" s="16"/>
@@ -35621,10 +35539,10 @@
     <row r="33" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A33" s="16"/>
       <c r="B33" s="42" t="s">
-        <v>68</v>
+        <v>57</v>
       </c>
       <c r="C33" s="16" t="s">
-        <v>69</v>
+        <v>58</v>
       </c>
       <c r="D33" s="16"/>
       <c r="E33" s="16"/>
@@ -35637,10 +35555,10 @@
     <row r="34" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A34" s="16"/>
       <c r="B34" s="42" t="s">
-        <v>70</v>
+        <v>59</v>
       </c>
       <c r="C34" s="16" t="s">
-        <v>71</v>
+        <v>60</v>
       </c>
       <c r="D34" s="16"/>
       <c r="E34" s="16"/>
@@ -35653,10 +35571,10 @@
     <row r="35" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A35" s="16"/>
       <c r="B35" s="42" t="s">
-        <v>72</v>
+        <v>61</v>
       </c>
       <c r="C35" s="16" t="s">
-        <v>73</v>
+        <v>62</v>
       </c>
       <c r="D35" s="16"/>
       <c r="E35" s="16"/>
@@ -35669,10 +35587,10 @@
     <row r="36" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A36" s="16"/>
       <c r="B36" s="42" t="s">
-        <v>74</v>
+        <v>63</v>
       </c>
       <c r="C36" s="39" t="s">
-        <v>75</v>
+        <v>64</v>
       </c>
       <c r="D36" s="16"/>
       <c r="E36" s="16"/>
@@ -35685,10 +35603,10 @@
     <row r="37" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A37" s="16"/>
       <c r="B37" s="42" t="s">
-        <v>76</v>
+        <v>65</v>
       </c>
       <c r="C37" s="16" t="s">
-        <v>77</v>
+        <v>66</v>
       </c>
       <c r="D37" s="16"/>
       <c r="E37" s="16"/>
@@ -35701,10 +35619,10 @@
     <row r="38" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A38" s="16"/>
       <c r="B38" s="42" t="s">
-        <v>78</v>
+        <v>67</v>
       </c>
       <c r="C38" s="16" t="s">
-        <v>79</v>
+        <v>68</v>
       </c>
       <c r="D38" s="16"/>
       <c r="E38" s="16"/>
@@ -35764,7 +35682,7 @@
     <row r="1" ht="39" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="43"/>
       <c r="B1" s="44" t="s">
-        <v>80</v>
+        <v>69</v>
       </c>
       <c r="C1" s="44"/>
       <c r="D1" s="44"/>
@@ -35784,20 +35702,20 @@
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="45"/>
       <c r="B3" s="45" t="s">
-        <v>81</v>
+        <v>70</v>
       </c>
       <c r="C3" s="45"/>
       <c r="D3" s="45"/>
       <c r="E3" s="45"/>
       <c r="F3" s="47" t="s">
-        <v>82</v>
+        <v>71</v>
       </c>
       <c r="G3" s="45"/>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="45"/>
       <c r="B4" s="45" t="s">
-        <v>83</v>
+        <v>72</v>
       </c>
       <c r="C4" s="45"/>
       <c r="D4" s="45"/>
@@ -35807,7 +35725,7 @@
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" s="43"/>
       <c r="B5" s="45" t="s">
-        <v>84</v>
+        <v>73</v>
       </c>
       <c r="C5" s="45"/>
       <c r="D5" s="45"/>
@@ -35827,35 +35745,35 @@
     <row r="7" ht="21.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" s="50"/>
       <c r="B7" s="51" t="s">
-        <v>85</v>
+        <v>74</v>
       </c>
       <c r="C7" s="52" t="s">
-        <v>86</v>
+        <v>75</v>
       </c>
       <c r="D7" s="52" t="s">
-        <v>87</v>
+        <v>76</v>
       </c>
       <c r="E7" s="52" t="s">
-        <v>88</v>
+        <v>77</v>
       </c>
       <c r="F7" s="53" t="s">
-        <v>89</v>
+        <v>78</v>
       </c>
       <c r="G7" s="54"/>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="50"/>
       <c r="B8" s="55" t="s">
-        <v>90</v>
+        <v>79</v>
       </c>
       <c r="C8" s="11" t="s">
-        <v>91</v>
+        <v>80</v>
       </c>
       <c r="D8" s="56" t="s">
-        <v>92</v>
+        <v>81</v>
       </c>
       <c r="E8" s="57" t="s">
-        <v>92</v>
+        <v>81</v>
       </c>
       <c r="F8" s="58"/>
       <c r="G8" s="54"/>
@@ -35863,16 +35781,16 @@
     <row r="9" ht="14.25" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="50"/>
       <c r="B9" s="59" t="s">
-        <v>93</v>
+        <v>82</v>
       </c>
       <c r="C9" s="60" t="s">
-        <v>94</v>
+        <v>83</v>
       </c>
       <c r="D9" s="56" t="s">
-        <v>92</v>
+        <v>81</v>
       </c>
       <c r="E9" s="61" t="s">
-        <v>92</v>
+        <v>81</v>
       </c>
       <c r="F9" s="62"/>
       <c r="G9" s="54"/>
@@ -35880,16 +35798,16 @@
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="50"/>
       <c r="B10" s="55" t="s">
-        <v>95</v>
+        <v>84</v>
       </c>
       <c r="C10" s="11" t="s">
-        <v>96</v>
+        <v>85</v>
       </c>
       <c r="D10" s="56" t="s">
-        <v>92</v>
+        <v>81</v>
       </c>
       <c r="E10" s="57" t="s">
-        <v>92</v>
+        <v>81</v>
       </c>
       <c r="F10" s="58"/>
       <c r="G10" s="54"/>
@@ -35900,13 +35818,13 @@
         <v>15</v>
       </c>
       <c r="C11" s="60" t="s">
-        <v>97</v>
+        <v>86</v>
       </c>
       <c r="D11" s="56" t="s">
-        <v>92</v>
+        <v>81</v>
       </c>
       <c r="E11" s="61" t="s">
-        <v>92</v>
+        <v>81</v>
       </c>
       <c r="F11" s="62"/>
       <c r="G11" s="54"/>
@@ -35914,16 +35832,16 @@
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" s="50"/>
       <c r="B12" s="55" t="s">
-        <v>98</v>
+        <v>87</v>
       </c>
       <c r="C12" s="11" t="s">
-        <v>99</v>
+        <v>88</v>
       </c>
       <c r="D12" s="56" t="s">
-        <v>92</v>
+        <v>81</v>
       </c>
       <c r="E12" s="57" t="s">
-        <v>92</v>
+        <v>81</v>
       </c>
       <c r="F12" s="58"/>
       <c r="G12" s="54"/>
@@ -35931,92 +35849,92 @@
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="50"/>
       <c r="B13" s="59" t="s">
-        <v>100</v>
+        <v>89</v>
       </c>
       <c r="C13" s="60" t="s">
-        <v>101</v>
+        <v>90</v>
       </c>
       <c r="D13" s="56" t="s">
-        <v>92</v>
+        <v>81</v>
       </c>
       <c r="E13" s="61" t="s">
-        <v>92</v>
+        <v>81</v>
       </c>
       <c r="F13" s="62" t="s">
-        <v>102</v>
+        <v>91</v>
       </c>
       <c r="G13" s="54"/>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" s="50"/>
       <c r="B14" s="55" t="s">
-        <v>103</v>
+        <v>92</v>
       </c>
       <c r="C14" s="11" t="s">
-        <v>104</v>
+        <v>93</v>
       </c>
       <c r="D14" s="56" t="s">
-        <v>92</v>
+        <v>81</v>
       </c>
       <c r="E14" s="57" t="s">
-        <v>92</v>
+        <v>81</v>
       </c>
       <c r="F14" s="58" t="s">
-        <v>102</v>
+        <v>91</v>
       </c>
       <c r="G14" s="54"/>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A15" s="50"/>
       <c r="B15" s="59" t="s">
-        <v>105</v>
+        <v>94</v>
       </c>
       <c r="C15" s="60" t="s">
-        <v>106</v>
+        <v>95</v>
       </c>
       <c r="D15" s="56" t="s">
-        <v>92</v>
+        <v>81</v>
       </c>
       <c r="E15" s="61" t="s">
-        <v>92</v>
+        <v>81</v>
       </c>
       <c r="F15" s="62" t="s">
-        <v>107</v>
+        <v>96</v>
       </c>
       <c r="G15" s="54"/>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" s="50"/>
       <c r="B16" s="55" t="s">
-        <v>108</v>
+        <v>97</v>
       </c>
       <c r="C16" s="11" t="s">
-        <v>109</v>
+        <v>98</v>
       </c>
       <c r="D16" s="56" t="s">
-        <v>92</v>
+        <v>81</v>
       </c>
       <c r="E16" s="57" t="s">
-        <v>92</v>
+        <v>81</v>
       </c>
       <c r="F16" s="58" t="s">
-        <v>107</v>
+        <v>96</v>
       </c>
       <c r="G16" s="54"/>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" s="50"/>
       <c r="B17" s="59" t="s">
-        <v>110</v>
+        <v>99</v>
       </c>
       <c r="C17" s="60" t="s">
-        <v>111</v>
+        <v>100</v>
       </c>
       <c r="D17" s="56" t="s">
-        <v>92</v>
+        <v>81</v>
       </c>
       <c r="E17" s="61" t="s">
-        <v>92</v>
+        <v>81</v>
       </c>
       <c r="F17" s="62"/>
       <c r="G17" s="54"/>
@@ -36024,16 +35942,16 @@
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" s="50"/>
       <c r="B18" s="55" t="s">
-        <v>112</v>
+        <v>101</v>
       </c>
       <c r="C18" s="11" t="s">
-        <v>113</v>
+        <v>102</v>
       </c>
       <c r="D18" s="56" t="s">
-        <v>92</v>
+        <v>81</v>
       </c>
       <c r="E18" s="57" t="s">
-        <v>92</v>
+        <v>81</v>
       </c>
       <c r="F18" s="58"/>
       <c r="G18" s="54"/>
@@ -36041,16 +35959,16 @@
     <row r="19" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A19" s="50"/>
       <c r="B19" s="59" t="s">
-        <v>114</v>
+        <v>103</v>
       </c>
       <c r="C19" s="60" t="s">
-        <v>115</v>
+        <v>104</v>
       </c>
       <c r="D19" s="56" t="s">
-        <v>92</v>
+        <v>81</v>
       </c>
       <c r="E19" s="61" t="s">
-        <v>92</v>
+        <v>81</v>
       </c>
       <c r="F19" s="62"/>
       <c r="G19" s="54"/>
@@ -36058,16 +35976,16 @@
     <row r="20" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A20" s="50"/>
       <c r="B20" s="55" t="s">
-        <v>116</v>
+        <v>105</v>
       </c>
       <c r="C20" s="11" t="s">
-        <v>117</v>
+        <v>106</v>
       </c>
       <c r="D20" s="56" t="s">
-        <v>92</v>
+        <v>81</v>
       </c>
       <c r="E20" s="57" t="s">
-        <v>92</v>
+        <v>81</v>
       </c>
       <c r="F20" s="58"/>
       <c r="G20" s="54"/>
@@ -36075,35 +35993,35 @@
     <row r="21" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A21" s="50"/>
       <c r="B21" s="59" t="s">
-        <v>118</v>
+        <v>107</v>
       </c>
       <c r="C21" s="60" t="s">
-        <v>119</v>
+        <v>108</v>
       </c>
       <c r="D21" s="56" t="s">
-        <v>92</v>
+        <v>81</v>
       </c>
       <c r="E21" s="61" t="s">
-        <v>92</v>
+        <v>81</v>
       </c>
       <c r="F21" s="63" t="s">
-        <v>120</v>
+        <v>109</v>
       </c>
       <c r="G21" s="54"/>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A22" s="50"/>
       <c r="B22" s="55" t="s">
-        <v>121</v>
+        <v>110</v>
       </c>
       <c r="C22" s="11" t="s">
-        <v>122</v>
+        <v>111</v>
       </c>
       <c r="D22" s="56" t="s">
-        <v>92</v>
+        <v>81</v>
       </c>
       <c r="E22" s="57" t="s">
-        <v>92</v>
+        <v>81</v>
       </c>
       <c r="F22" s="58"/>
       <c r="G22" s="54"/>
@@ -36111,16 +36029,16 @@
     <row r="23" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A23" s="50"/>
       <c r="B23" s="59" t="s">
-        <v>123</v>
+        <v>112</v>
       </c>
       <c r="C23" s="60" t="s">
-        <v>124</v>
+        <v>113</v>
       </c>
       <c r="D23" s="56" t="s">
-        <v>92</v>
+        <v>81</v>
       </c>
       <c r="E23" s="61" t="s">
-        <v>92</v>
+        <v>81</v>
       </c>
       <c r="F23" s="62"/>
       <c r="G23" s="54"/>
@@ -36128,16 +36046,16 @@
     <row r="24" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A24" s="50"/>
       <c r="B24" s="64" t="s">
-        <v>125</v>
+        <v>114</v>
       </c>
       <c r="C24" s="11" t="s">
-        <v>126</v>
+        <v>115</v>
       </c>
       <c r="D24" s="65" t="s">
-        <v>92</v>
+        <v>81</v>
       </c>
       <c r="E24" s="66" t="s">
-        <v>92</v>
+        <v>81</v>
       </c>
       <c r="F24" s="67"/>
       <c r="G24" s="68"/>
@@ -36145,19 +36063,19 @@
     <row r="25" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A25" s="50"/>
       <c r="B25" s="59" t="s">
-        <v>127</v>
+        <v>116</v>
       </c>
       <c r="C25" s="60" t="s">
-        <v>128</v>
+        <v>117</v>
       </c>
       <c r="D25" s="56" t="s">
-        <v>92</v>
+        <v>81</v>
       </c>
       <c r="E25" s="61" t="s">
-        <v>92</v>
+        <v>81</v>
       </c>
       <c r="F25" s="62" t="s">
-        <v>129</v>
+        <v>118</v>
       </c>
       <c r="G25" s="69"/>
     </row>
@@ -36167,32 +36085,32 @@
         <v>16</v>
       </c>
       <c r="C26" s="11" t="s">
-        <v>130</v>
+        <v>119</v>
       </c>
       <c r="D26" s="56" t="s">
-        <v>92</v>
+        <v>81</v>
       </c>
       <c r="E26" s="57" t="s">
-        <v>92</v>
+        <v>81</v>
       </c>
       <c r="F26" s="58" t="s">
-        <v>131</v>
+        <v>120</v>
       </c>
       <c r="G26" s="54"/>
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A27" s="50"/>
       <c r="B27" s="59" t="s">
-        <v>132</v>
+        <v>121</v>
       </c>
       <c r="C27" s="60" t="s">
-        <v>133</v>
+        <v>122</v>
       </c>
       <c r="D27" s="56" t="s">
-        <v>92</v>
+        <v>81</v>
       </c>
       <c r="E27" s="61" t="s">
-        <v>134</v>
+        <v>123</v>
       </c>
       <c r="F27" s="62"/>
       <c r="G27" s="54"/>
@@ -36200,38 +36118,38 @@
     <row r="28" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A28" s="50"/>
       <c r="B28" s="55" t="s">
-        <v>135</v>
+        <v>124</v>
       </c>
       <c r="C28" s="11" t="s">
-        <v>136</v>
+        <v>125</v>
       </c>
       <c r="D28" s="56" t="s">
-        <v>92</v>
+        <v>81</v>
       </c>
       <c r="E28" s="57" t="s">
-        <v>92</v>
+        <v>81</v>
       </c>
       <c r="F28" s="67" t="s">
-        <v>137</v>
+        <v>126</v>
       </c>
       <c r="G28" s="54"/>
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A29" s="50"/>
       <c r="B29" s="59" t="s">
-        <v>138</v>
+        <v>127</v>
       </c>
       <c r="C29" s="60" t="s">
-        <v>139</v>
+        <v>128</v>
       </c>
       <c r="D29" s="56" t="s">
-        <v>92</v>
+        <v>81</v>
       </c>
       <c r="E29" s="61" t="s">
-        <v>134</v>
+        <v>123</v>
       </c>
       <c r="F29" s="62" t="s">
-        <v>140</v>
+        <v>129</v>
       </c>
       <c r="G29" s="54"/>
     </row>
@@ -36241,13 +36159,13 @@
         <v>18</v>
       </c>
       <c r="C30" s="11" t="s">
-        <v>141</v>
+        <v>130</v>
       </c>
       <c r="D30" s="56" t="s">
-        <v>92</v>
+        <v>81</v>
       </c>
       <c r="E30" s="57" t="s">
-        <v>92</v>
+        <v>81</v>
       </c>
       <c r="F30" s="58"/>
       <c r="G30" s="54"/>
@@ -36255,16 +36173,16 @@
     <row r="31" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A31" s="50"/>
       <c r="B31" s="59" t="s">
-        <v>142</v>
+        <v>131</v>
       </c>
       <c r="C31" s="60" t="s">
-        <v>143</v>
+        <v>132</v>
       </c>
       <c r="D31" s="56" t="s">
-        <v>92</v>
+        <v>81</v>
       </c>
       <c r="E31" s="61" t="s">
-        <v>92</v>
+        <v>81</v>
       </c>
       <c r="F31" s="62"/>
       <c r="G31" s="54"/>
@@ -36272,16 +36190,16 @@
     <row r="32" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A32" s="50"/>
       <c r="B32" s="55" t="s">
-        <v>144</v>
+        <v>133</v>
       </c>
       <c r="C32" s="11" t="s">
-        <v>145</v>
+        <v>134</v>
       </c>
       <c r="D32" s="56" t="s">
-        <v>92</v>
+        <v>81</v>
       </c>
       <c r="E32" s="57" t="s">
-        <v>92</v>
+        <v>81</v>
       </c>
       <c r="F32" s="58"/>
       <c r="G32" s="54"/>
@@ -36289,16 +36207,16 @@
     <row r="33" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A33" s="50"/>
       <c r="B33" s="59" t="s">
-        <v>146</v>
+        <v>135</v>
       </c>
       <c r="C33" s="60" t="s">
-        <v>147</v>
+        <v>136</v>
       </c>
       <c r="D33" s="56" t="s">
-        <v>92</v>
+        <v>81</v>
       </c>
       <c r="E33" s="61" t="s">
-        <v>92</v>
+        <v>81</v>
       </c>
       <c r="F33" s="62"/>
       <c r="G33" s="54"/>
@@ -36306,16 +36224,16 @@
     <row r="34" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A34" s="50"/>
       <c r="B34" s="55" t="s">
-        <v>148</v>
+        <v>137</v>
       </c>
       <c r="C34" s="11" t="s">
-        <v>149</v>
+        <v>138</v>
       </c>
       <c r="D34" s="56" t="s">
-        <v>92</v>
+        <v>81</v>
       </c>
       <c r="E34" s="57" t="s">
-        <v>92</v>
+        <v>81</v>
       </c>
       <c r="F34" s="58"/>
       <c r="G34" s="54"/>
@@ -36323,16 +36241,16 @@
     <row r="35" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A35" s="50"/>
       <c r="B35" s="59" t="s">
-        <v>150</v>
+        <v>139</v>
       </c>
       <c r="C35" s="60" t="s">
-        <v>151</v>
+        <v>140</v>
       </c>
       <c r="D35" s="56" t="s">
-        <v>92</v>
+        <v>81</v>
       </c>
       <c r="E35" s="61" t="s">
-        <v>92</v>
+        <v>81</v>
       </c>
       <c r="F35" s="62"/>
       <c r="G35" s="54"/>
@@ -36340,16 +36258,16 @@
     <row r="36" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A36" s="50"/>
       <c r="B36" s="55" t="s">
-        <v>152</v>
+        <v>141</v>
       </c>
       <c r="C36" s="11" t="s">
-        <v>153</v>
+        <v>142</v>
       </c>
       <c r="D36" s="56" t="s">
-        <v>92</v>
+        <v>81</v>
       </c>
       <c r="E36" s="57" t="s">
-        <v>92</v>
+        <v>81</v>
       </c>
       <c r="F36" s="58"/>
       <c r="G36" s="54"/>
@@ -36357,16 +36275,16 @@
     <row r="37" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A37" s="50"/>
       <c r="B37" s="59" t="s">
-        <v>154</v>
+        <v>143</v>
       </c>
       <c r="C37" s="60" t="s">
-        <v>155</v>
+        <v>144</v>
       </c>
       <c r="D37" s="56" t="s">
-        <v>92</v>
+        <v>81</v>
       </c>
       <c r="E37" s="61" t="s">
-        <v>92</v>
+        <v>81</v>
       </c>
       <c r="F37" s="62"/>
       <c r="G37" s="54"/>
@@ -36374,16 +36292,16 @@
     <row r="38" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A38" s="50"/>
       <c r="B38" s="55" t="s">
-        <v>156</v>
+        <v>145</v>
       </c>
       <c r="C38" s="11" t="s">
-        <v>157</v>
+        <v>146</v>
       </c>
       <c r="D38" s="56" t="s">
-        <v>92</v>
+        <v>81</v>
       </c>
       <c r="E38" s="57" t="s">
-        <v>92</v>
+        <v>81</v>
       </c>
       <c r="F38" s="58"/>
       <c r="G38" s="54"/>
@@ -36391,16 +36309,16 @@
     <row r="39" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A39" s="50"/>
       <c r="B39" s="59" t="s">
-        <v>158</v>
+        <v>147</v>
       </c>
       <c r="C39" s="60" t="s">
-        <v>159</v>
+        <v>148</v>
       </c>
       <c r="D39" s="56" t="s">
-        <v>92</v>
+        <v>81</v>
       </c>
       <c r="E39" s="61" t="s">
-        <v>92</v>
+        <v>81</v>
       </c>
       <c r="F39" s="62"/>
       <c r="G39" s="54"/>
@@ -36408,16 +36326,16 @@
     <row r="40" ht="21.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A40" s="50"/>
       <c r="B40" s="55" t="s">
-        <v>160</v>
+        <v>149</v>
       </c>
       <c r="C40" s="11" t="s">
-        <v>161</v>
+        <v>150</v>
       </c>
       <c r="D40" s="56" t="s">
-        <v>92</v>
+        <v>81</v>
       </c>
       <c r="E40" s="57" t="s">
-        <v>92</v>
+        <v>81</v>
       </c>
       <c r="F40" s="58"/>
       <c r="G40" s="54"/>
@@ -36425,16 +36343,16 @@
     <row r="41" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A41" s="50"/>
       <c r="B41" s="59" t="s">
-        <v>162</v>
+        <v>151</v>
       </c>
       <c r="C41" s="60" t="s">
-        <v>163</v>
+        <v>152</v>
       </c>
       <c r="D41" s="56" t="s">
-        <v>92</v>
+        <v>81</v>
       </c>
       <c r="E41" s="61" t="s">
-        <v>92</v>
+        <v>81</v>
       </c>
       <c r="F41" s="62"/>
       <c r="G41" s="54"/>
@@ -36442,16 +36360,16 @@
     <row r="42" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A42" s="50"/>
       <c r="B42" s="55" t="s">
-        <v>164</v>
+        <v>153</v>
       </c>
       <c r="C42" s="11" t="s">
-        <v>165</v>
+        <v>154</v>
       </c>
       <c r="D42" s="56" t="s">
-        <v>92</v>
+        <v>81</v>
       </c>
       <c r="E42" s="57" t="s">
-        <v>92</v>
+        <v>81</v>
       </c>
       <c r="F42" s="58"/>
       <c r="G42" s="54"/>
@@ -36459,16 +36377,16 @@
     <row r="43" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A43" s="50"/>
       <c r="B43" s="59" t="s">
-        <v>166</v>
+        <v>155</v>
       </c>
       <c r="C43" s="60" t="s">
-        <v>167</v>
+        <v>156</v>
       </c>
       <c r="D43" s="56" t="s">
-        <v>92</v>
+        <v>81</v>
       </c>
       <c r="E43" s="61" t="s">
-        <v>134</v>
+        <v>123</v>
       </c>
       <c r="F43" s="70"/>
       <c r="G43" s="54"/>
@@ -36476,16 +36394,16 @@
     <row r="44" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A44" s="50"/>
       <c r="B44" s="55" t="s">
-        <v>168</v>
+        <v>157</v>
       </c>
       <c r="C44" s="11" t="s">
-        <v>169</v>
+        <v>158</v>
       </c>
       <c r="D44" s="56" t="s">
-        <v>92</v>
+        <v>81</v>
       </c>
       <c r="E44" s="57" t="s">
-        <v>134</v>
+        <v>123</v>
       </c>
       <c r="F44" s="71"/>
       <c r="G44" s="54"/>
@@ -36493,16 +36411,16 @@
     <row r="45" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A45" s="72"/>
       <c r="B45" s="59" t="s">
-        <v>170</v>
+        <v>159</v>
       </c>
       <c r="C45" s="60" t="s">
-        <v>171</v>
+        <v>160</v>
       </c>
       <c r="D45" s="56" t="s">
-        <v>92</v>
+        <v>81</v>
       </c>
       <c r="E45" s="61" t="s">
-        <v>92</v>
+        <v>81</v>
       </c>
       <c r="F45" s="62"/>
       <c r="G45" s="54"/>
@@ -36510,19 +36428,19 @@
     <row r="46" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A46" s="50"/>
       <c r="B46" s="73" t="s">
-        <v>172</v>
+        <v>161</v>
       </c>
       <c r="C46" s="74" t="s">
-        <v>173</v>
+        <v>162</v>
       </c>
       <c r="D46" s="75" t="s">
-        <v>92</v>
+        <v>81</v>
       </c>
       <c r="E46" s="76" t="s">
-        <v>134</v>
+        <v>123</v>
       </c>
       <c r="F46" s="77" t="s">
-        <v>174</v>
+        <v>163</v>
       </c>
       <c r="G46" s="54"/>
     </row>
@@ -36566,7 +36484,7 @@
     <row r="1" ht="41.25" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="80"/>
       <c r="B1" s="44" t="s">
-        <v>175</v>
+        <v>164</v>
       </c>
       <c r="C1" s="44"/>
       <c r="D1" s="44"/>
@@ -36586,7 +36504,7 @@
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="81"/>
       <c r="B3" s="45" t="s">
-        <v>176</v>
+        <v>165</v>
       </c>
       <c r="C3" s="81"/>
       <c r="D3" s="81"/>
@@ -36597,7 +36515,7 @@
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="81"/>
       <c r="B4" s="45" t="s">
-        <v>177</v>
+        <v>166</v>
       </c>
       <c r="C4" s="81"/>
       <c r="D4" s="81"/>
@@ -36617,741 +36535,741 @@
     <row r="6" ht="25.5" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" s="84"/>
       <c r="B6" s="51" t="s">
-        <v>178</v>
+        <v>167</v>
       </c>
       <c r="C6" s="52" t="s">
-        <v>86</v>
+        <v>75</v>
       </c>
       <c r="D6" s="52" t="s">
-        <v>179</v>
+        <v>168</v>
       </c>
       <c r="E6" s="52" t="s">
-        <v>87</v>
+        <v>76</v>
       </c>
       <c r="F6" s="85" t="s">
-        <v>88</v>
+        <v>77</v>
       </c>
       <c r="G6" s="86"/>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" s="82"/>
       <c r="B7" s="55" t="s">
-        <v>180</v>
+        <v>169</v>
       </c>
       <c r="C7" s="87" t="s">
-        <v>181</v>
+        <v>170</v>
       </c>
       <c r="D7" s="87" t="s">
-        <v>90</v>
+        <v>79</v>
       </c>
       <c r="E7" s="57" t="s">
-        <v>92</v>
+        <v>81</v>
       </c>
       <c r="F7" s="88" t="s">
-        <v>182</v>
+        <v>171</v>
       </c>
       <c r="G7" s="86"/>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="82"/>
       <c r="B8" s="59" t="s">
-        <v>183</v>
+        <v>172</v>
       </c>
       <c r="C8" s="89" t="s">
-        <v>184</v>
+        <v>173</v>
       </c>
       <c r="D8" s="89" t="s">
-        <v>90</v>
+        <v>79</v>
       </c>
       <c r="E8" s="90" t="s">
-        <v>185</v>
+        <v>174</v>
       </c>
       <c r="F8" s="91" t="s">
-        <v>92</v>
+        <v>81</v>
       </c>
       <c r="G8" s="92"/>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="82"/>
       <c r="B9" s="55" t="s">
-        <v>186</v>
+        <v>175</v>
       </c>
       <c r="C9" s="87" t="s">
-        <v>187</v>
+        <v>176</v>
       </c>
       <c r="D9" s="87" t="s">
-        <v>90</v>
+        <v>79</v>
       </c>
       <c r="E9" s="57" t="s">
-        <v>92</v>
+        <v>81</v>
       </c>
       <c r="F9" s="88" t="s">
-        <v>92</v>
+        <v>81</v>
       </c>
       <c r="G9" s="86"/>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="82"/>
       <c r="B10" s="59" t="s">
-        <v>188</v>
+        <v>177</v>
       </c>
       <c r="C10" s="60" t="s">
-        <v>189</v>
+        <v>178</v>
       </c>
       <c r="D10" s="60" t="s">
-        <v>190</v>
+        <v>179</v>
       </c>
       <c r="E10" s="61" t="s">
-        <v>92</v>
+        <v>81</v>
       </c>
       <c r="F10" s="91" t="s">
-        <v>134</v>
+        <v>123</v>
       </c>
       <c r="G10" s="86"/>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="93"/>
       <c r="B11" s="64" t="s">
-        <v>191</v>
+        <v>180</v>
       </c>
       <c r="C11" s="11" t="s">
-        <v>192</v>
+        <v>181</v>
       </c>
       <c r="D11" s="11" t="s">
-        <v>193</v>
+        <v>182</v>
       </c>
       <c r="E11" s="66" t="s">
-        <v>92</v>
+        <v>81</v>
       </c>
       <c r="F11" s="94" t="s">
-        <v>92</v>
+        <v>81</v>
       </c>
       <c r="G11" s="95"/>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" s="82"/>
       <c r="B12" s="59" t="s">
-        <v>194</v>
+        <v>183</v>
       </c>
       <c r="C12" s="89" t="s">
-        <v>195</v>
+        <v>184</v>
       </c>
       <c r="D12" s="89" t="s">
-        <v>95</v>
+        <v>84</v>
       </c>
       <c r="E12" s="61" t="s">
-        <v>92</v>
+        <v>81</v>
       </c>
       <c r="F12" s="91" t="s">
-        <v>134</v>
+        <v>123</v>
       </c>
       <c r="G12" s="86"/>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="82"/>
       <c r="B13" s="55" t="s">
-        <v>196</v>
+        <v>185</v>
       </c>
       <c r="C13" s="87" t="s">
-        <v>197</v>
+        <v>186</v>
       </c>
       <c r="D13" s="87" t="s">
-        <v>127</v>
+        <v>116</v>
       </c>
       <c r="E13" s="57" t="s">
-        <v>92</v>
+        <v>81</v>
       </c>
       <c r="F13" s="88" t="s">
-        <v>92</v>
+        <v>81</v>
       </c>
       <c r="G13" s="86"/>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" s="82"/>
       <c r="B14" s="59" t="s">
-        <v>198</v>
+        <v>187</v>
       </c>
       <c r="C14" s="89" t="s">
-        <v>199</v>
+        <v>188</v>
       </c>
       <c r="D14" s="89" t="s">
-        <v>127</v>
+        <v>116</v>
       </c>
       <c r="E14" s="61" t="s">
-        <v>92</v>
+        <v>81</v>
       </c>
       <c r="F14" s="91" t="s">
-        <v>92</v>
+        <v>81</v>
       </c>
       <c r="G14" s="86"/>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A15" s="82"/>
       <c r="B15" s="55" t="s">
-        <v>200</v>
+        <v>189</v>
       </c>
       <c r="C15" s="87" t="s">
-        <v>201</v>
+        <v>190</v>
       </c>
       <c r="D15" s="87" t="s">
-        <v>127</v>
+        <v>116</v>
       </c>
       <c r="E15" s="57" t="s">
-        <v>92</v>
+        <v>81</v>
       </c>
       <c r="F15" s="88" t="s">
-        <v>92</v>
+        <v>81</v>
       </c>
       <c r="G15" s="86"/>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" s="82"/>
       <c r="B16" s="59" t="s">
-        <v>202</v>
+        <v>191</v>
       </c>
       <c r="C16" s="89" t="s">
-        <v>203</v>
+        <v>192</v>
       </c>
       <c r="D16" s="89" t="s">
-        <v>127</v>
+        <v>116</v>
       </c>
       <c r="E16" s="61" t="s">
-        <v>92</v>
+        <v>81</v>
       </c>
       <c r="F16" s="91" t="s">
-        <v>92</v>
+        <v>81</v>
       </c>
       <c r="G16" s="86"/>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" s="82"/>
       <c r="B17" s="55" t="s">
-        <v>204</v>
+        <v>193</v>
       </c>
       <c r="C17" s="87" t="s">
-        <v>205</v>
+        <v>194</v>
       </c>
       <c r="D17" s="87" t="s">
-        <v>206</v>
+        <v>195</v>
       </c>
       <c r="E17" s="57" t="s">
-        <v>92</v>
+        <v>81</v>
       </c>
       <c r="F17" s="88" t="s">
-        <v>182</v>
+        <v>171</v>
       </c>
       <c r="G17" s="86"/>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" s="82"/>
       <c r="B18" s="59" t="s">
-        <v>207</v>
+        <v>196</v>
       </c>
       <c r="C18" s="89" t="s">
-        <v>208</v>
+        <v>197</v>
       </c>
       <c r="D18" s="89" t="s">
         <v>16</v>
       </c>
       <c r="E18" s="61" t="s">
-        <v>92</v>
+        <v>81</v>
       </c>
       <c r="F18" s="91" t="s">
-        <v>182</v>
+        <v>171</v>
       </c>
       <c r="G18" s="86"/>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A19" s="82"/>
       <c r="B19" s="55" t="s">
-        <v>209</v>
+        <v>198</v>
       </c>
       <c r="C19" s="87" t="s">
-        <v>210</v>
+        <v>199</v>
       </c>
       <c r="D19" s="87" t="s">
         <v>16</v>
       </c>
       <c r="E19" s="57" t="s">
-        <v>92</v>
+        <v>81</v>
       </c>
       <c r="F19" s="88" t="s">
-        <v>92</v>
+        <v>81</v>
       </c>
       <c r="G19" s="86"/>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A20" s="82"/>
       <c r="B20" s="59" t="s">
-        <v>211</v>
+        <v>200</v>
       </c>
       <c r="C20" s="89" t="s">
-        <v>212</v>
+        <v>201</v>
       </c>
       <c r="D20" s="89" t="s">
         <v>16</v>
       </c>
       <c r="E20" s="61" t="s">
-        <v>92</v>
+        <v>81</v>
       </c>
       <c r="F20" s="91" t="s">
-        <v>92</v>
+        <v>81</v>
       </c>
       <c r="G20" s="86"/>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A21" s="82"/>
       <c r="B21" s="55" t="s">
-        <v>213</v>
+        <v>202</v>
       </c>
       <c r="C21" s="87" t="s">
-        <v>214</v>
+        <v>203</v>
       </c>
       <c r="D21" s="87" t="s">
         <v>16</v>
       </c>
       <c r="E21" s="57" t="s">
-        <v>92</v>
+        <v>81</v>
       </c>
       <c r="F21" s="88" t="s">
-        <v>92</v>
+        <v>81</v>
       </c>
       <c r="G21" s="86"/>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A22" s="82"/>
       <c r="B22" s="59" t="s">
-        <v>215</v>
+        <v>204</v>
       </c>
       <c r="C22" s="89" t="s">
-        <v>216</v>
+        <v>205</v>
       </c>
       <c r="D22" s="89" t="s">
-        <v>217</v>
+        <v>206</v>
       </c>
       <c r="E22" s="61" t="s">
-        <v>92</v>
+        <v>81</v>
       </c>
       <c r="F22" s="91" t="s">
-        <v>134</v>
+        <v>123</v>
       </c>
       <c r="G22" s="86"/>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A23" s="82"/>
       <c r="B23" s="55" t="s">
-        <v>218</v>
+        <v>207</v>
       </c>
       <c r="C23" s="87" t="s">
-        <v>219</v>
+        <v>208</v>
       </c>
       <c r="D23" s="87" t="s">
-        <v>144</v>
+        <v>133</v>
       </c>
       <c r="E23" s="57" t="s">
-        <v>92</v>
+        <v>81</v>
       </c>
       <c r="F23" s="88" t="s">
-        <v>182</v>
+        <v>171</v>
       </c>
       <c r="G23" s="86"/>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A24" s="82"/>
       <c r="B24" s="59" t="s">
-        <v>220</v>
+        <v>209</v>
       </c>
       <c r="C24" s="89" t="s">
-        <v>221</v>
+        <v>210</v>
       </c>
       <c r="D24" s="89" t="s">
-        <v>144</v>
+        <v>133</v>
       </c>
       <c r="E24" s="61" t="s">
-        <v>92</v>
+        <v>81</v>
       </c>
       <c r="F24" s="91" t="s">
-        <v>222</v>
+        <v>211</v>
       </c>
       <c r="G24" s="86"/>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A25" s="82"/>
       <c r="B25" s="55" t="s">
-        <v>223</v>
+        <v>212</v>
       </c>
       <c r="C25" s="87" t="s">
-        <v>224</v>
+        <v>213</v>
       </c>
       <c r="D25" s="87" t="s">
-        <v>144</v>
+        <v>133</v>
       </c>
       <c r="E25" s="57" t="s">
-        <v>92</v>
+        <v>81</v>
       </c>
       <c r="F25" s="88" t="s">
-        <v>134</v>
+        <v>123</v>
       </c>
       <c r="G25" s="86"/>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A26" s="82"/>
       <c r="B26" s="59" t="s">
-        <v>225</v>
+        <v>214</v>
       </c>
       <c r="C26" s="89" t="s">
-        <v>226</v>
+        <v>215</v>
       </c>
       <c r="D26" s="89" t="s">
-        <v>144</v>
+        <v>133</v>
       </c>
       <c r="E26" s="61" t="s">
-        <v>92</v>
+        <v>81</v>
       </c>
       <c r="F26" s="91" t="s">
-        <v>134</v>
+        <v>123</v>
       </c>
       <c r="G26" s="86"/>
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A27" s="82"/>
       <c r="B27" s="55" t="s">
-        <v>227</v>
+        <v>216</v>
       </c>
       <c r="C27" s="87" t="s">
-        <v>228</v>
+        <v>217</v>
       </c>
       <c r="D27" s="87" t="s">
-        <v>144</v>
+        <v>133</v>
       </c>
       <c r="E27" s="57" t="s">
-        <v>92</v>
+        <v>81</v>
       </c>
       <c r="F27" s="88" t="s">
-        <v>134</v>
+        <v>123</v>
       </c>
       <c r="G27" s="86"/>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A28" s="82"/>
       <c r="B28" s="59" t="s">
-        <v>229</v>
+        <v>218</v>
       </c>
       <c r="C28" s="89" t="s">
-        <v>230</v>
+        <v>219</v>
       </c>
       <c r="D28" s="89" t="s">
-        <v>144</v>
+        <v>133</v>
       </c>
       <c r="E28" s="61" t="s">
-        <v>92</v>
+        <v>81</v>
       </c>
       <c r="F28" s="91" t="s">
-        <v>134</v>
+        <v>123</v>
       </c>
       <c r="G28" s="86"/>
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A29" s="82"/>
       <c r="B29" s="55" t="s">
-        <v>231</v>
+        <v>220</v>
       </c>
       <c r="C29" s="87" t="s">
-        <v>232</v>
+        <v>221</v>
       </c>
       <c r="D29" s="87" t="s">
-        <v>144</v>
+        <v>133</v>
       </c>
       <c r="E29" s="57" t="s">
-        <v>92</v>
+        <v>81</v>
       </c>
       <c r="F29" s="88" t="s">
-        <v>134</v>
+        <v>123</v>
       </c>
       <c r="G29" s="86"/>
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A30" s="82"/>
       <c r="B30" s="59" t="s">
-        <v>233</v>
+        <v>222</v>
       </c>
       <c r="C30" s="89" t="s">
-        <v>234</v>
+        <v>223</v>
       </c>
       <c r="D30" s="89" t="s">
-        <v>144</v>
+        <v>133</v>
       </c>
       <c r="E30" s="61" t="s">
-        <v>92</v>
+        <v>81</v>
       </c>
       <c r="F30" s="91" t="s">
-        <v>134</v>
+        <v>123</v>
       </c>
       <c r="G30" s="86"/>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A31" s="82"/>
       <c r="B31" s="55" t="s">
-        <v>235</v>
+        <v>224</v>
       </c>
       <c r="C31" s="87" t="s">
-        <v>236</v>
+        <v>225</v>
       </c>
       <c r="D31" s="87" t="s">
-        <v>118</v>
+        <v>107</v>
       </c>
       <c r="E31" s="57" t="s">
-        <v>92</v>
+        <v>81</v>
       </c>
       <c r="F31" s="88" t="s">
-        <v>92</v>
+        <v>81</v>
       </c>
       <c r="G31" s="86"/>
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A32" s="82"/>
       <c r="B32" s="59" t="s">
-        <v>237</v>
+        <v>226</v>
       </c>
       <c r="C32" s="60" t="s">
-        <v>238</v>
+        <v>227</v>
       </c>
       <c r="D32" s="89" t="s">
-        <v>118</v>
+        <v>107</v>
       </c>
       <c r="E32" s="61" t="s">
-        <v>92</v>
+        <v>81</v>
       </c>
       <c r="F32" s="91" t="s">
-        <v>92</v>
+        <v>81</v>
       </c>
       <c r="G32" s="86"/>
     </row>
     <row r="33" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A33" s="82"/>
       <c r="B33" s="55" t="s">
-        <v>239</v>
+        <v>228</v>
       </c>
       <c r="C33" s="87" t="s">
-        <v>240</v>
+        <v>229</v>
       </c>
       <c r="D33" s="87" t="s">
-        <v>241</v>
+        <v>230</v>
       </c>
       <c r="E33" s="57" t="s">
-        <v>242</v>
+        <v>231</v>
       </c>
       <c r="F33" s="88" t="s">
-        <v>92</v>
+        <v>81</v>
       </c>
       <c r="G33" s="86"/>
     </row>
     <row r="34" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A34" s="82"/>
       <c r="B34" s="59" t="s">
-        <v>243</v>
+        <v>232</v>
       </c>
       <c r="C34" s="89" t="s">
-        <v>244</v>
+        <v>233</v>
       </c>
       <c r="D34" s="89" t="s">
-        <v>245</v>
+        <v>234</v>
       </c>
       <c r="E34" s="61" t="s">
-        <v>92</v>
+        <v>81</v>
       </c>
       <c r="F34" s="91" t="s">
-        <v>92</v>
+        <v>81</v>
       </c>
       <c r="G34" s="86"/>
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A35" s="82"/>
       <c r="B35" s="55" t="s">
-        <v>246</v>
+        <v>235</v>
       </c>
       <c r="C35" s="87" t="s">
-        <v>247</v>
+        <v>236</v>
       </c>
       <c r="D35" s="87" t="s">
-        <v>245</v>
+        <v>234</v>
       </c>
       <c r="E35" s="57" t="s">
-        <v>92</v>
+        <v>81</v>
       </c>
       <c r="F35" s="88" t="s">
-        <v>248</v>
+        <v>237</v>
       </c>
       <c r="G35" s="86"/>
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A36" s="82"/>
       <c r="B36" s="59" t="s">
-        <v>249</v>
+        <v>238</v>
       </c>
       <c r="C36" s="89" t="s">
-        <v>250</v>
+        <v>239</v>
       </c>
       <c r="D36" s="89" t="s">
-        <v>251</v>
+        <v>240</v>
       </c>
       <c r="E36" s="61" t="s">
-        <v>92</v>
+        <v>81</v>
       </c>
       <c r="F36" s="91" t="s">
-        <v>134</v>
+        <v>123</v>
       </c>
       <c r="G36" s="86"/>
     </row>
     <row r="37" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A37" s="82"/>
       <c r="B37" s="55" t="s">
-        <v>252</v>
+        <v>241</v>
       </c>
       <c r="C37" s="87" t="s">
-        <v>253</v>
+        <v>242</v>
       </c>
       <c r="D37" s="87" t="s">
-        <v>245</v>
+        <v>234</v>
       </c>
       <c r="E37" s="57" t="s">
-        <v>92</v>
+        <v>81</v>
       </c>
       <c r="F37" s="88" t="s">
-        <v>92</v>
+        <v>81</v>
       </c>
       <c r="G37" s="86"/>
     </row>
     <row r="38" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A38" s="82"/>
       <c r="B38" s="59" t="s">
-        <v>254</v>
+        <v>243</v>
       </c>
       <c r="C38" s="60" t="s">
-        <v>255</v>
+        <v>244</v>
       </c>
       <c r="D38" s="89" t="s">
-        <v>245</v>
+        <v>234</v>
       </c>
       <c r="E38" s="61" t="s">
-        <v>92</v>
+        <v>81</v>
       </c>
       <c r="F38" s="91" t="s">
-        <v>92</v>
+        <v>81</v>
       </c>
       <c r="G38" s="86"/>
     </row>
     <row r="39" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A39" s="82"/>
       <c r="B39" s="55" t="s">
-        <v>256</v>
+        <v>245</v>
       </c>
       <c r="C39" s="87" t="s">
-        <v>257</v>
+        <v>246</v>
       </c>
       <c r="D39" s="87" t="s">
-        <v>245</v>
+        <v>234</v>
       </c>
       <c r="E39" s="57" t="s">
-        <v>92</v>
+        <v>81</v>
       </c>
       <c r="F39" s="88" t="s">
-        <v>92</v>
+        <v>81</v>
       </c>
       <c r="G39" s="86"/>
     </row>
     <row r="40" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A40" s="82"/>
       <c r="B40" s="59" t="s">
-        <v>258</v>
+        <v>247</v>
       </c>
       <c r="C40" s="89" t="s">
-        <v>259</v>
+        <v>248</v>
       </c>
       <c r="D40" s="89" t="s">
-        <v>245</v>
+        <v>234</v>
       </c>
       <c r="E40" s="61" t="s">
-        <v>92</v>
+        <v>81</v>
       </c>
       <c r="F40" s="91" t="s">
-        <v>92</v>
+        <v>81</v>
       </c>
       <c r="G40" s="86"/>
     </row>
     <row r="41" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A41" s="82"/>
       <c r="B41" s="55" t="s">
-        <v>260</v>
+        <v>249</v>
       </c>
       <c r="C41" s="11" t="s">
-        <v>261</v>
+        <v>250</v>
       </c>
       <c r="D41" s="87" t="s">
-        <v>245</v>
+        <v>234</v>
       </c>
       <c r="E41" s="57" t="s">
-        <v>92</v>
+        <v>81</v>
       </c>
       <c r="F41" s="88" t="s">
-        <v>92</v>
+        <v>81</v>
       </c>
       <c r="G41" s="86"/>
     </row>
     <row r="42" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A42" s="82"/>
       <c r="B42" s="59" t="s">
-        <v>262</v>
+        <v>251</v>
       </c>
       <c r="C42" s="89" t="s">
-        <v>263</v>
+        <v>252</v>
       </c>
       <c r="D42" s="89" t="s">
-        <v>251</v>
+        <v>240</v>
       </c>
       <c r="E42" s="61" t="s">
-        <v>92</v>
+        <v>81</v>
       </c>
       <c r="F42" s="91" t="s">
-        <v>92</v>
+        <v>81</v>
       </c>
       <c r="G42" s="86"/>
     </row>
     <row r="43" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A43" s="82"/>
       <c r="B43" s="55" t="s">
-        <v>264</v>
+        <v>253</v>
       </c>
       <c r="C43" s="11" t="s">
-        <v>265</v>
+        <v>254</v>
       </c>
       <c r="D43" s="87" t="s">
-        <v>251</v>
+        <v>240</v>
       </c>
       <c r="E43" s="57" t="s">
-        <v>92</v>
+        <v>81</v>
       </c>
       <c r="F43" s="88" t="s">
-        <v>134</v>
+        <v>123</v>
       </c>
       <c r="G43" s="86"/>
     </row>
     <row r="44" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A44" s="82"/>
       <c r="B44" s="59" t="s">
-        <v>266</v>
+        <v>255</v>
       </c>
       <c r="C44" s="89" t="s">
-        <v>267</v>
+        <v>256</v>
       </c>
       <c r="D44" s="89" t="s">
-        <v>268</v>
+        <v>257</v>
       </c>
       <c r="E44" s="61" t="s">
-        <v>92</v>
+        <v>81</v>
       </c>
       <c r="F44" s="96" t="s">
-        <v>269</v>
+        <v>258</v>
       </c>
       <c r="G44" s="86"/>
     </row>
@@ -37361,149 +37279,149 @@
         <v>2</v>
       </c>
       <c r="C45" s="87" t="s">
-        <v>270</v>
+        <v>259</v>
       </c>
       <c r="D45" s="87" t="s">
-        <v>245</v>
+        <v>234</v>
       </c>
       <c r="E45" s="57" t="s">
-        <v>92</v>
+        <v>81</v>
       </c>
       <c r="F45" s="88" t="s">
-        <v>92</v>
+        <v>81</v>
       </c>
       <c r="G45" s="86"/>
     </row>
     <row r="46" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A46" s="82"/>
       <c r="B46" s="59" t="s">
-        <v>271</v>
+        <v>260</v>
       </c>
       <c r="C46" s="89" t="s">
-        <v>272</v>
+        <v>261</v>
       </c>
       <c r="D46" s="89" t="s">
-        <v>245</v>
+        <v>234</v>
       </c>
       <c r="E46" s="61" t="s">
-        <v>92</v>
+        <v>81</v>
       </c>
       <c r="F46" s="91" t="s">
-        <v>92</v>
+        <v>81</v>
       </c>
       <c r="G46" s="86"/>
     </row>
     <row r="47" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A47" s="82"/>
       <c r="B47" s="73" t="s">
-        <v>273</v>
+        <v>262</v>
       </c>
       <c r="C47" s="97" t="s">
-        <v>274</v>
+        <v>263</v>
       </c>
       <c r="D47" s="97" t="s">
-        <v>245</v>
+        <v>234</v>
       </c>
       <c r="E47" s="76" t="s">
-        <v>92</v>
+        <v>81</v>
       </c>
       <c r="F47" s="98" t="s">
-        <v>92</v>
+        <v>81</v>
       </c>
       <c r="G47" s="86"/>
     </row>
     <row r="48" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A48" s="99"/>
       <c r="B48" s="89" t="s">
-        <v>275</v>
+        <v>264</v>
       </c>
       <c r="C48" s="89" t="s">
-        <v>276</v>
+        <v>265</v>
       </c>
       <c r="D48" s="89" t="s">
-        <v>114</v>
+        <v>103</v>
       </c>
       <c r="E48" s="61" t="s">
-        <v>92</v>
+        <v>81</v>
       </c>
       <c r="F48" s="61" t="s">
-        <v>92</v>
+        <v>81</v>
       </c>
       <c r="G48" s="86"/>
     </row>
     <row r="49" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A49" s="82"/>
       <c r="B49" s="87" t="s">
-        <v>277</v>
+        <v>266</v>
       </c>
       <c r="C49" s="87" t="s">
-        <v>278</v>
+        <v>267</v>
       </c>
       <c r="D49" s="87" t="s">
-        <v>132</v>
+        <v>121</v>
       </c>
       <c r="E49" s="57" t="s">
-        <v>92</v>
+        <v>81</v>
       </c>
       <c r="F49" s="57" t="s">
-        <v>134</v>
+        <v>123</v>
       </c>
       <c r="G49" s="86"/>
     </row>
     <row r="50" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A50" s="99"/>
       <c r="B50" s="89" t="s">
-        <v>279</v>
+        <v>268</v>
       </c>
       <c r="C50" s="89" t="s">
-        <v>280</v>
+        <v>269</v>
       </c>
       <c r="D50" s="89" t="s">
-        <v>90</v>
+        <v>79</v>
       </c>
       <c r="E50" s="100" t="s">
-        <v>92</v>
+        <v>81</v>
       </c>
       <c r="F50" s="101" t="s">
-        <v>134</v>
+        <v>123</v>
       </c>
       <c r="G50" s="86"/>
     </row>
     <row r="51" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A51" s="82"/>
       <c r="B51" s="87" t="s">
-        <v>281</v>
+        <v>270</v>
       </c>
       <c r="C51" s="87" t="s">
-        <v>282</v>
+        <v>271</v>
       </c>
       <c r="D51" s="87" t="s">
-        <v>90</v>
+        <v>79</v>
       </c>
       <c r="E51" s="100" t="s">
-        <v>92</v>
+        <v>81</v>
       </c>
       <c r="F51" s="101" t="s">
-        <v>134</v>
+        <v>123</v>
       </c>
       <c r="G51" s="86"/>
     </row>
     <row r="52" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A52" s="99"/>
       <c r="B52" s="89" t="s">
-        <v>283</v>
+        <v>272</v>
       </c>
       <c r="C52" s="89" t="s">
-        <v>284</v>
+        <v>273</v>
       </c>
       <c r="D52" s="89" t="s">
-        <v>93</v>
+        <v>82</v>
       </c>
       <c r="E52" s="100" t="s">
-        <v>92</v>
+        <v>81</v>
       </c>
       <c r="F52" s="101" t="s">
-        <v>134</v>
+        <v>123</v>
       </c>
       <c r="G52" s="86"/>
     </row>
@@ -37540,7 +37458,7 @@
     <row r="1" ht="39.75" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="103"/>
       <c r="B1" s="44" t="s">
-        <v>285</v>
+        <v>274</v>
       </c>
       <c r="C1" s="44"/>
       <c r="D1" s="104"/>
@@ -37554,7 +37472,7 @@
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="81"/>
       <c r="B3" s="45" t="s">
-        <v>286</v>
+        <v>275</v>
       </c>
       <c r="C3" s="81"/>
       <c r="D3" s="81"/>
@@ -37562,7 +37480,7 @@
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" s="81"/>
       <c r="B4" s="45" t="s">
-        <v>287</v>
+        <v>276</v>
       </c>
       <c r="C4" s="81"/>
       <c r="D4" s="81"/>
@@ -37570,7 +37488,7 @@
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" s="81"/>
       <c r="B5" s="45" t="s">
-        <v>288</v>
+        <v>277</v>
       </c>
       <c r="C5" s="81"/>
       <c r="D5" s="81"/>
@@ -37578,7 +37496,7 @@
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" s="81"/>
       <c r="B6" s="47" t="s">
-        <v>289</v>
+        <v>278</v>
       </c>
       <c r="C6" s="81"/>
       <c r="D6" s="81"/>
@@ -37592,110 +37510,110 @@
     <row r="8" ht="24" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" s="93"/>
       <c r="B8" s="105" t="s">
-        <v>290</v>
+        <v>279</v>
       </c>
       <c r="C8" s="106" t="s">
-        <v>86</v>
+        <v>75</v>
       </c>
       <c r="D8" s="86"/>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" s="93"/>
       <c r="B9" s="64" t="s">
-        <v>291</v>
+        <v>280</v>
       </c>
       <c r="C9" s="107" t="s">
-        <v>292</v>
+        <v>281</v>
       </c>
       <c r="D9" s="86"/>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" s="93"/>
       <c r="B10" s="64" t="s">
-        <v>293</v>
+        <v>282</v>
       </c>
       <c r="C10" s="107" t="s">
-        <v>294</v>
+        <v>283</v>
       </c>
       <c r="D10" s="86"/>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" s="93"/>
       <c r="B11" s="64" t="s">
-        <v>295</v>
+        <v>284</v>
       </c>
       <c r="C11" s="107" t="s">
-        <v>296</v>
+        <v>285</v>
       </c>
       <c r="D11" s="86"/>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" s="93"/>
       <c r="B12" s="64" t="s">
-        <v>297</v>
+        <v>286</v>
       </c>
       <c r="C12" s="107" t="s">
-        <v>298</v>
+        <v>287</v>
       </c>
       <c r="D12" s="86"/>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13" s="93"/>
       <c r="B13" s="64" t="s">
-        <v>299</v>
+        <v>288</v>
       </c>
       <c r="C13" s="107" t="s">
-        <v>300</v>
+        <v>289</v>
       </c>
       <c r="D13" s="86"/>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14" s="93"/>
       <c r="B14" s="64" t="s">
-        <v>301</v>
+        <v>290</v>
       </c>
       <c r="C14" s="107" t="s">
-        <v>302</v>
+        <v>291</v>
       </c>
       <c r="D14" s="86"/>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A15" s="93"/>
       <c r="B15" s="64" t="s">
-        <v>303</v>
+        <v>292</v>
       </c>
       <c r="C15" s="107" t="s">
-        <v>304</v>
+        <v>293</v>
       </c>
       <c r="D15" s="86"/>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A16" s="93"/>
       <c r="B16" s="64" t="s">
-        <v>305</v>
+        <v>294</v>
       </c>
       <c r="C16" s="107" t="s">
-        <v>306</v>
+        <v>295</v>
       </c>
       <c r="D16" s="86"/>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A17" s="93"/>
       <c r="B17" s="64" t="s">
-        <v>307</v>
+        <v>296</v>
       </c>
       <c r="C17" s="107" t="s">
-        <v>308</v>
+        <v>297</v>
       </c>
       <c r="D17" s="86"/>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A18" s="93"/>
       <c r="B18" s="108" t="s">
-        <v>309</v>
+        <v>298</v>
       </c>
       <c r="C18" s="109" t="s">
-        <v>310</v>
+        <v>299</v>
       </c>
       <c r="D18" s="86"/>
     </row>
@@ -37730,7 +37648,7 @@
     <row r="1" ht="38.25" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="80"/>
       <c r="B1" s="44" t="s">
-        <v>311</v>
+        <v>300</v>
       </c>
       <c r="C1" s="44"/>
       <c r="D1" s="81"/>
@@ -37744,7 +37662,7 @@
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="81"/>
       <c r="B3" s="81" t="s">
-        <v>312</v>
+        <v>301</v>
       </c>
       <c r="C3" s="81"/>
       <c r="D3" s="81"/>
@@ -37752,7 +37670,7 @@
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" s="81"/>
       <c r="B4" s="81" t="s">
-        <v>313</v>
+        <v>302</v>
       </c>
       <c r="C4" s="81"/>
       <c r="D4" s="81"/>
@@ -37760,7 +37678,7 @@
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" s="81"/>
       <c r="B5" s="110" t="s">
-        <v>314</v>
+        <v>303</v>
       </c>
       <c r="C5" s="81"/>
       <c r="D5" s="81"/>
@@ -37774,150 +37692,150 @@
     <row r="7" ht="21.75" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" s="111"/>
       <c r="B7" s="112" t="s">
-        <v>315</v>
+        <v>304</v>
       </c>
       <c r="C7" s="113" t="s">
-        <v>86</v>
+        <v>75</v>
       </c>
       <c r="D7" s="86"/>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" s="82"/>
       <c r="B8" s="114" t="s">
-        <v>316</v>
+        <v>305</v>
       </c>
       <c r="C8" s="115" t="s">
-        <v>317</v>
+        <v>306</v>
       </c>
       <c r="D8" s="86"/>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" s="82"/>
       <c r="B9" s="114" t="s">
-        <v>318</v>
+        <v>307</v>
       </c>
       <c r="C9" s="115" t="s">
-        <v>319</v>
+        <v>308</v>
       </c>
       <c r="D9" s="86"/>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" s="82"/>
       <c r="B10" s="114" t="s">
-        <v>320</v>
+        <v>309</v>
       </c>
       <c r="C10" s="115" t="s">
-        <v>321</v>
+        <v>310</v>
       </c>
       <c r="D10" s="86"/>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" s="82"/>
       <c r="B11" s="114" t="s">
-        <v>322</v>
+        <v>311</v>
       </c>
       <c r="C11" s="115" t="s">
-        <v>323</v>
+        <v>312</v>
       </c>
       <c r="D11" s="86"/>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" s="82"/>
       <c r="B12" s="114" t="s">
-        <v>324</v>
+        <v>313</v>
       </c>
       <c r="C12" s="115" t="s">
-        <v>325</v>
+        <v>314</v>
       </c>
       <c r="D12" s="86"/>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13" s="82"/>
       <c r="B13" s="114" t="s">
-        <v>326</v>
+        <v>315</v>
       </c>
       <c r="C13" s="115" t="s">
-        <v>327</v>
+        <v>316</v>
       </c>
       <c r="D13" s="86"/>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14" s="82"/>
       <c r="B14" s="114" t="s">
-        <v>328</v>
+        <v>317</v>
       </c>
       <c r="C14" s="115" t="s">
-        <v>329</v>
+        <v>318</v>
       </c>
       <c r="D14" s="86"/>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A15" s="82"/>
       <c r="B15" s="114" t="s">
-        <v>330</v>
+        <v>319</v>
       </c>
       <c r="C15" s="115" t="s">
-        <v>331</v>
+        <v>320</v>
       </c>
       <c r="D15" s="86"/>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A16" s="82"/>
       <c r="B16" s="114" t="s">
-        <v>332</v>
+        <v>321</v>
       </c>
       <c r="C16" s="115" t="s">
-        <v>333</v>
+        <v>322</v>
       </c>
       <c r="D16" s="86"/>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A17" s="82"/>
       <c r="B17" s="114" t="s">
-        <v>334</v>
+        <v>323</v>
       </c>
       <c r="C17" s="115" t="s">
-        <v>335</v>
+        <v>324</v>
       </c>
       <c r="D17" s="86"/>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A18" s="82"/>
       <c r="B18" s="114" t="s">
-        <v>336</v>
+        <v>325</v>
       </c>
       <c r="C18" s="115" t="s">
-        <v>337</v>
+        <v>326</v>
       </c>
       <c r="D18" s="86"/>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A19" s="82"/>
       <c r="B19" s="114" t="s">
-        <v>338</v>
+        <v>327</v>
       </c>
       <c r="C19" s="116" t="s">
-        <v>339</v>
+        <v>328</v>
       </c>
       <c r="D19" s="86"/>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A20" s="82"/>
       <c r="B20" s="114" t="s">
-        <v>340</v>
+        <v>329</v>
       </c>
       <c r="C20" s="115" t="s">
-        <v>341</v>
+        <v>330</v>
       </c>
       <c r="D20" s="86"/>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A21" s="82"/>
       <c r="B21" s="117" t="s">
-        <v>342</v>
+        <v>331</v>
       </c>
       <c r="C21" s="118" t="s">
-        <v>343</v>
+        <v>332</v>
       </c>
       <c r="D21" s="86"/>
     </row>

</xml_diff>